<commit_message>
Basic data & prep app limits
</commit_message>
<xml_diff>
--- a/resources/TierPlus Planning.xlsx
+++ b/resources/TierPlus Planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="509" documentId="8_{E97B7BBA-A1CF-CA4D-89B6-D5BE4B7D4A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66925795-9227-CF46-89C9-CE763E0B4A2F}"/>
+  <xr:revisionPtr revIDLastSave="532" documentId="8_{E97B7BBA-A1CF-CA4D-89B6-D5BE4B7D4A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F401DFC-54D7-6345-9741-7BC40F98E887}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
   <si>
     <t>Project start:</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>Define assumptions for baseline interventions in the abscence of data</t>
+  </si>
+  <si>
+    <t>Need a check for if I'm missing things</t>
   </si>
 </sst>
 </file>
@@ -843,7 +846,7 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1142,6 +1145,29 @@
     <xf numFmtId="0" fontId="19" fillId="5" borderId="8" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="19" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1163,28 +1189,8 @@
     <xf numFmtId="166" fontId="19" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -2048,7 +2054,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="15" fmlaLink="$Q$2" horiz="1" max="100" page="0" val="6"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="15" fmlaLink="$Q$2" horiz="1" max="100" page="0"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2381,8 +2387,8 @@
     <col min="4" max="4" width="10.6640625" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" style="106" customWidth="1"/>
     <col min="6" max="6" width="6.6640625" style="107" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2.6640625" customWidth="1"/>
-    <col min="8" max="8" width="6" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.6640625" customWidth="1"/>
     <col min="9" max="92" width="2.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2396,29 +2402,28 @@
       <c r="E1" s="82"/>
       <c r="F1" s="83"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="116" t="s">
+      <c r="I1" s="125" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="126"/>
       <c r="P1" s="18"/>
-      <c r="Q1" s="114">
-        <f ca="1">TODAY()</f>
+      <c r="Q1" s="123">
         <v>46064</v>
       </c>
-      <c r="R1" s="115"/>
-      <c r="S1" s="115"/>
-      <c r="T1" s="115"/>
-      <c r="U1" s="115"/>
-      <c r="V1" s="115"/>
-      <c r="W1" s="115"/>
-      <c r="X1" s="115"/>
-      <c r="Y1" s="115"/>
-      <c r="Z1" s="115"/>
+      <c r="R1" s="124"/>
+      <c r="S1" s="124"/>
+      <c r="T1" s="124"/>
+      <c r="U1" s="124"/>
+      <c r="V1" s="124"/>
+      <c r="W1" s="124"/>
+      <c r="X1" s="124"/>
+      <c r="Y1" s="124"/>
+      <c r="Z1" s="124"/>
     </row>
     <row r="2" spans="1:92" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="71"/>
@@ -2428,28 +2433,28 @@
       <c r="D2" s="17"/>
       <c r="E2" s="84"/>
       <c r="F2" s="85"/>
-      <c r="I2" s="116" t="s">
+      <c r="I2" s="125" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="117"/>
-      <c r="K2" s="117"/>
-      <c r="L2" s="117"/>
-      <c r="M2" s="117"/>
-      <c r="N2" s="117"/>
-      <c r="O2" s="117"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
+      <c r="O2" s="126"/>
       <c r="P2" s="18"/>
-      <c r="Q2" s="112">
-        <v>6</v>
-      </c>
-      <c r="R2" s="113"/>
-      <c r="S2" s="113"/>
-      <c r="T2" s="113"/>
-      <c r="U2" s="113"/>
-      <c r="V2" s="113"/>
-      <c r="W2" s="113"/>
-      <c r="X2" s="113"/>
-      <c r="Y2" s="113"/>
-      <c r="Z2" s="113"/>
+      <c r="Q2" s="121">
+        <v>1</v>
+      </c>
+      <c r="R2" s="122"/>
+      <c r="S2" s="122"/>
+      <c r="T2" s="122"/>
+      <c r="U2" s="122"/>
+      <c r="V2" s="122"/>
+      <c r="W2" s="122"/>
+      <c r="X2" s="122"/>
+      <c r="Y2" s="122"/>
+      <c r="Z2" s="122"/>
       <c r="AP2" t="s">
         <v>63</v>
       </c>
@@ -2463,827 +2468,827 @@
     </row>
     <row r="4" spans="1:92" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="81"/>
-      <c r="B4" s="127" t="s">
+      <c r="B4" s="110" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="88"/>
       <c r="F4" s="87"/>
-      <c r="I4" s="118">
-        <f ca="1">I5</f>
+      <c r="I4" s="127">
+        <f>I5</f>
+        <v>46062</v>
+      </c>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="119">
+        <f>P5</f>
+        <v>46069</v>
+      </c>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
+      <c r="U4" s="119"/>
+      <c r="V4" s="119"/>
+      <c r="W4" s="119">
+        <f>W5</f>
+        <v>46076</v>
+      </c>
+      <c r="X4" s="119"/>
+      <c r="Y4" s="119"/>
+      <c r="Z4" s="119"/>
+      <c r="AA4" s="119"/>
+      <c r="AB4" s="119"/>
+      <c r="AC4" s="119"/>
+      <c r="AD4" s="119">
+        <f>AD5</f>
+        <v>46083</v>
+      </c>
+      <c r="AE4" s="119"/>
+      <c r="AF4" s="119"/>
+      <c r="AG4" s="119"/>
+      <c r="AH4" s="119"/>
+      <c r="AI4" s="119"/>
+      <c r="AJ4" s="119"/>
+      <c r="AK4" s="119">
+        <f>AK5</f>
+        <v>46090</v>
+      </c>
+      <c r="AL4" s="119"/>
+      <c r="AM4" s="119"/>
+      <c r="AN4" s="119"/>
+      <c r="AO4" s="119"/>
+      <c r="AP4" s="119"/>
+      <c r="AQ4" s="119"/>
+      <c r="AR4" s="119">
+        <f>AR5</f>
         <v>46097</v>
       </c>
-      <c r="J4" s="110"/>
-      <c r="K4" s="110"/>
-      <c r="L4" s="110"/>
-      <c r="M4" s="110"/>
-      <c r="N4" s="110"/>
-      <c r="O4" s="110"/>
-      <c r="P4" s="110">
-        <f ca="1">P5</f>
+      <c r="AS4" s="119"/>
+      <c r="AT4" s="119"/>
+      <c r="AU4" s="119"/>
+      <c r="AV4" s="119"/>
+      <c r="AW4" s="119"/>
+      <c r="AX4" s="119"/>
+      <c r="AY4" s="119">
+        <f>AY5</f>
         <v>46104</v>
       </c>
-      <c r="Q4" s="110"/>
-      <c r="R4" s="110"/>
-      <c r="S4" s="110"/>
-      <c r="T4" s="110"/>
-      <c r="U4" s="110"/>
-      <c r="V4" s="110"/>
-      <c r="W4" s="110">
-        <f ca="1">W5</f>
+      <c r="AZ4" s="119"/>
+      <c r="BA4" s="119"/>
+      <c r="BB4" s="119"/>
+      <c r="BC4" s="119"/>
+      <c r="BD4" s="119"/>
+      <c r="BE4" s="119"/>
+      <c r="BF4" s="119">
+        <f>BF5</f>
         <v>46111</v>
       </c>
-      <c r="X4" s="110"/>
-      <c r="Y4" s="110"/>
-      <c r="Z4" s="110"/>
-      <c r="AA4" s="110"/>
-      <c r="AB4" s="110"/>
-      <c r="AC4" s="110"/>
-      <c r="AD4" s="110">
-        <f ca="1">AD5</f>
+      <c r="BG4" s="119"/>
+      <c r="BH4" s="119"/>
+      <c r="BI4" s="119"/>
+      <c r="BJ4" s="119"/>
+      <c r="BK4" s="119"/>
+      <c r="BL4" s="120"/>
+      <c r="BM4" s="119">
+        <f>BM5</f>
         <v>46118</v>
       </c>
-      <c r="AE4" s="110"/>
-      <c r="AF4" s="110"/>
-      <c r="AG4" s="110"/>
-      <c r="AH4" s="110"/>
-      <c r="AI4" s="110"/>
-      <c r="AJ4" s="110"/>
-      <c r="AK4" s="110">
-        <f ca="1">AK5</f>
+      <c r="BN4" s="119"/>
+      <c r="BO4" s="119"/>
+      <c r="BP4" s="119"/>
+      <c r="BQ4" s="119"/>
+      <c r="BR4" s="119"/>
+      <c r="BS4" s="120"/>
+      <c r="BT4" s="119">
+        <f>BT5</f>
         <v>46125</v>
       </c>
-      <c r="AL4" s="110"/>
-      <c r="AM4" s="110"/>
-      <c r="AN4" s="110"/>
-      <c r="AO4" s="110"/>
-      <c r="AP4" s="110"/>
-      <c r="AQ4" s="110"/>
-      <c r="AR4" s="110">
-        <f ca="1">AR5</f>
+      <c r="BU4" s="119"/>
+      <c r="BV4" s="119"/>
+      <c r="BW4" s="119"/>
+      <c r="BX4" s="119"/>
+      <c r="BY4" s="119"/>
+      <c r="BZ4" s="120"/>
+      <c r="CA4" s="119">
+        <f>CA5</f>
         <v>46132</v>
       </c>
-      <c r="AS4" s="110"/>
-      <c r="AT4" s="110"/>
-      <c r="AU4" s="110"/>
-      <c r="AV4" s="110"/>
-      <c r="AW4" s="110"/>
-      <c r="AX4" s="110"/>
-      <c r="AY4" s="110">
-        <f ca="1">AY5</f>
+      <c r="CB4" s="119"/>
+      <c r="CC4" s="119"/>
+      <c r="CD4" s="119"/>
+      <c r="CE4" s="119"/>
+      <c r="CF4" s="119"/>
+      <c r="CG4" s="120"/>
+      <c r="CH4" s="119">
+        <f>CH5</f>
         <v>46139</v>
       </c>
-      <c r="AZ4" s="110"/>
-      <c r="BA4" s="110"/>
-      <c r="BB4" s="110"/>
-      <c r="BC4" s="110"/>
-      <c r="BD4" s="110"/>
-      <c r="BE4" s="110"/>
-      <c r="BF4" s="110">
-        <f ca="1">BF5</f>
-        <v>46146</v>
-      </c>
-      <c r="BG4" s="110"/>
-      <c r="BH4" s="110"/>
-      <c r="BI4" s="110"/>
-      <c r="BJ4" s="110"/>
-      <c r="BK4" s="110"/>
-      <c r="BL4" s="111"/>
-      <c r="BM4" s="110">
-        <f ca="1">BM5</f>
-        <v>46153</v>
-      </c>
-      <c r="BN4" s="110"/>
-      <c r="BO4" s="110"/>
-      <c r="BP4" s="110"/>
-      <c r="BQ4" s="110"/>
-      <c r="BR4" s="110"/>
-      <c r="BS4" s="111"/>
-      <c r="BT4" s="110">
-        <f ca="1">BT5</f>
-        <v>46160</v>
-      </c>
-      <c r="BU4" s="110"/>
-      <c r="BV4" s="110"/>
-      <c r="BW4" s="110"/>
-      <c r="BX4" s="110"/>
-      <c r="BY4" s="110"/>
-      <c r="BZ4" s="111"/>
-      <c r="CA4" s="110">
-        <f ca="1">CA5</f>
-        <v>46167</v>
-      </c>
-      <c r="CB4" s="110"/>
-      <c r="CC4" s="110"/>
-      <c r="CD4" s="110"/>
-      <c r="CE4" s="110"/>
-      <c r="CF4" s="110"/>
-      <c r="CG4" s="111"/>
-      <c r="CH4" s="110">
-        <f ca="1">CH5</f>
-        <v>46174</v>
-      </c>
-      <c r="CI4" s="110"/>
-      <c r="CJ4" s="110"/>
-      <c r="CK4" s="110"/>
-      <c r="CL4" s="110"/>
-      <c r="CM4" s="110"/>
-      <c r="CN4" s="111"/>
+      <c r="CI4" s="119"/>
+      <c r="CJ4" s="119"/>
+      <c r="CK4" s="119"/>
+      <c r="CL4" s="119"/>
+      <c r="CM4" s="119"/>
+      <c r="CN4" s="120"/>
     </row>
     <row r="5" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="119"/>
-      <c r="B5" s="120" t="s">
+      <c r="A5" s="113"/>
+      <c r="B5" s="114" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="122" t="s">
+      <c r="C5" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="124" t="s">
+      <c r="D5" s="118" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="125" t="s">
+      <c r="E5" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="125" t="s">
+      <c r="F5" s="111" t="s">
         <v>9</v>
       </c>
       <c r="I5" s="22">
-        <f ca="1">Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
+        <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
+        <v>46062</v>
+      </c>
+      <c r="J5" s="22">
+        <f>I5+1</f>
+        <v>46063</v>
+      </c>
+      <c r="K5" s="22">
+        <f t="shared" ref="K5:AX5" si="0">J5+1</f>
+        <v>46064</v>
+      </c>
+      <c r="L5" s="22">
+        <f t="shared" si="0"/>
+        <v>46065</v>
+      </c>
+      <c r="M5" s="22">
+        <f t="shared" si="0"/>
+        <v>46066</v>
+      </c>
+      <c r="N5" s="22">
+        <f t="shared" si="0"/>
+        <v>46067</v>
+      </c>
+      <c r="O5" s="23">
+        <f t="shared" si="0"/>
+        <v>46068</v>
+      </c>
+      <c r="P5" s="24">
+        <f>O5+1</f>
+        <v>46069</v>
+      </c>
+      <c r="Q5" s="22">
+        <f>P5+1</f>
+        <v>46070</v>
+      </c>
+      <c r="R5" s="22">
+        <f t="shared" si="0"/>
+        <v>46071</v>
+      </c>
+      <c r="S5" s="22">
+        <f t="shared" si="0"/>
+        <v>46072</v>
+      </c>
+      <c r="T5" s="22">
+        <f t="shared" si="0"/>
+        <v>46073</v>
+      </c>
+      <c r="U5" s="22">
+        <f t="shared" si="0"/>
+        <v>46074</v>
+      </c>
+      <c r="V5" s="23">
+        <f t="shared" si="0"/>
+        <v>46075</v>
+      </c>
+      <c r="W5" s="24">
+        <f>V5+1</f>
+        <v>46076</v>
+      </c>
+      <c r="X5" s="22">
+        <f>W5+1</f>
+        <v>46077</v>
+      </c>
+      <c r="Y5" s="22">
+        <f t="shared" si="0"/>
+        <v>46078</v>
+      </c>
+      <c r="Z5" s="22">
+        <f t="shared" si="0"/>
+        <v>46079</v>
+      </c>
+      <c r="AA5" s="22">
+        <f t="shared" si="0"/>
+        <v>46080</v>
+      </c>
+      <c r="AB5" s="22">
+        <f t="shared" si="0"/>
+        <v>46081</v>
+      </c>
+      <c r="AC5" s="23">
+        <f t="shared" si="0"/>
+        <v>46082</v>
+      </c>
+      <c r="AD5" s="24">
+        <f>AC5+1</f>
+        <v>46083</v>
+      </c>
+      <c r="AE5" s="22">
+        <f>AD5+1</f>
+        <v>46084</v>
+      </c>
+      <c r="AF5" s="22">
+        <f t="shared" si="0"/>
+        <v>46085</v>
+      </c>
+      <c r="AG5" s="22">
+        <f t="shared" si="0"/>
+        <v>46086</v>
+      </c>
+      <c r="AH5" s="22">
+        <f t="shared" si="0"/>
+        <v>46087</v>
+      </c>
+      <c r="AI5" s="22">
+        <f t="shared" si="0"/>
+        <v>46088</v>
+      </c>
+      <c r="AJ5" s="23">
+        <f t="shared" si="0"/>
+        <v>46089</v>
+      </c>
+      <c r="AK5" s="24">
+        <f>AJ5+1</f>
+        <v>46090</v>
+      </c>
+      <c r="AL5" s="22">
+        <f>AK5+1</f>
+        <v>46091</v>
+      </c>
+      <c r="AM5" s="22">
+        <f t="shared" si="0"/>
+        <v>46092</v>
+      </c>
+      <c r="AN5" s="22">
+        <f t="shared" si="0"/>
+        <v>46093</v>
+      </c>
+      <c r="AO5" s="22">
+        <f t="shared" si="0"/>
+        <v>46094</v>
+      </c>
+      <c r="AP5" s="22">
+        <f t="shared" si="0"/>
+        <v>46095</v>
+      </c>
+      <c r="AQ5" s="23">
+        <f t="shared" si="0"/>
+        <v>46096</v>
+      </c>
+      <c r="AR5" s="24">
+        <f>AQ5+1</f>
         <v>46097</v>
       </c>
-      <c r="J5" s="22">
-        <f ca="1">I5+1</f>
+      <c r="AS5" s="22">
+        <f>AR5+1</f>
         <v>46098</v>
       </c>
-      <c r="K5" s="22">
-        <f t="shared" ref="K5:AX5" ca="1" si="0">J5+1</f>
+      <c r="AT5" s="22">
+        <f t="shared" si="0"/>
         <v>46099</v>
       </c>
-      <c r="L5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AU5" s="22">
+        <f t="shared" si="0"/>
         <v>46100</v>
       </c>
-      <c r="M5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AV5" s="22">
+        <f t="shared" si="0"/>
         <v>46101</v>
       </c>
-      <c r="N5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AW5" s="22">
+        <f t="shared" si="0"/>
         <v>46102</v>
       </c>
-      <c r="O5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AX5" s="23">
+        <f t="shared" si="0"/>
         <v>46103</v>
       </c>
-      <c r="P5" s="24">
-        <f ca="1">O5+1</f>
+      <c r="AY5" s="24">
+        <f>AX5+1</f>
         <v>46104</v>
       </c>
-      <c r="Q5" s="22">
-        <f ca="1">P5+1</f>
+      <c r="AZ5" s="22">
+        <f>AY5+1</f>
         <v>46105</v>
       </c>
-      <c r="R5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BA5" s="22">
+        <f t="shared" ref="BA5:BE5" si="1">AZ5+1</f>
         <v>46106</v>
       </c>
-      <c r="S5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BB5" s="22">
+        <f t="shared" si="1"/>
         <v>46107</v>
       </c>
-      <c r="T5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BC5" s="22">
+        <f t="shared" si="1"/>
         <v>46108</v>
       </c>
-      <c r="U5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BD5" s="22">
+        <f t="shared" si="1"/>
         <v>46109</v>
       </c>
-      <c r="V5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BE5" s="23">
+        <f t="shared" si="1"/>
         <v>46110</v>
       </c>
-      <c r="W5" s="24">
-        <f ca="1">V5+1</f>
+      <c r="BF5" s="24">
+        <f>BE5+1</f>
         <v>46111</v>
       </c>
-      <c r="X5" s="22">
-        <f ca="1">W5+1</f>
+      <c r="BG5" s="22">
+        <f>BF5+1</f>
         <v>46112</v>
       </c>
-      <c r="Y5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BH5" s="22">
+        <f t="shared" ref="BH5:BL5" si="2">BG5+1</f>
         <v>46113</v>
       </c>
-      <c r="Z5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BI5" s="22">
+        <f t="shared" si="2"/>
         <v>46114</v>
       </c>
-      <c r="AA5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BJ5" s="22">
+        <f t="shared" si="2"/>
         <v>46115</v>
       </c>
-      <c r="AB5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BK5" s="22">
+        <f t="shared" si="2"/>
         <v>46116</v>
       </c>
-      <c r="AC5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BL5" s="22">
+        <f t="shared" si="2"/>
         <v>46117</v>
       </c>
-      <c r="AD5" s="24">
-        <f ca="1">AC5+1</f>
+      <c r="BM5" s="24">
+        <f>BL5+1</f>
         <v>46118</v>
       </c>
-      <c r="AE5" s="22">
-        <f ca="1">AD5+1</f>
+      <c r="BN5" s="22">
+        <f>BM5+1</f>
         <v>46119</v>
       </c>
-      <c r="AF5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BO5" s="22">
+        <f t="shared" ref="BO5" si="3">BN5+1</f>
         <v>46120</v>
       </c>
-      <c r="AG5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BP5" s="22">
+        <f t="shared" ref="BP5" si="4">BO5+1</f>
         <v>46121</v>
       </c>
-      <c r="AH5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BQ5" s="22">
+        <f t="shared" ref="BQ5" si="5">BP5+1</f>
         <v>46122</v>
       </c>
-      <c r="AI5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BR5" s="22">
+        <f t="shared" ref="BR5" si="6">BQ5+1</f>
         <v>46123</v>
       </c>
-      <c r="AJ5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BS5" s="22">
+        <f t="shared" ref="BS5" si="7">BR5+1</f>
         <v>46124</v>
       </c>
-      <c r="AK5" s="24">
-        <f ca="1">AJ5+1</f>
+      <c r="BT5" s="24">
+        <f>BS5+1</f>
         <v>46125</v>
       </c>
-      <c r="AL5" s="22">
-        <f ca="1">AK5+1</f>
+      <c r="BU5" s="22">
+        <f>BT5+1</f>
         <v>46126</v>
       </c>
-      <c r="AM5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BV5" s="22">
+        <f t="shared" ref="BV5" si="8">BU5+1</f>
         <v>46127</v>
       </c>
-      <c r="AN5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BW5" s="22">
+        <f t="shared" ref="BW5" si="9">BV5+1</f>
         <v>46128</v>
       </c>
-      <c r="AO5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BX5" s="22">
+        <f t="shared" ref="BX5" si="10">BW5+1</f>
         <v>46129</v>
       </c>
-      <c r="AP5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BY5" s="22">
+        <f t="shared" ref="BY5" si="11">BX5+1</f>
         <v>46130</v>
       </c>
-      <c r="AQ5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BZ5" s="22">
+        <f t="shared" ref="BZ5" si="12">BY5+1</f>
         <v>46131</v>
       </c>
-      <c r="AR5" s="24">
-        <f ca="1">AQ5+1</f>
+      <c r="CA5" s="24">
+        <f>BZ5+1</f>
         <v>46132</v>
       </c>
-      <c r="AS5" s="22">
-        <f ca="1">AR5+1</f>
+      <c r="CB5" s="22">
+        <f>CA5+1</f>
         <v>46133</v>
       </c>
-      <c r="AT5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="CC5" s="22">
+        <f t="shared" ref="CC5" si="13">CB5+1</f>
         <v>46134</v>
       </c>
-      <c r="AU5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="CD5" s="22">
+        <f t="shared" ref="CD5" si="14">CC5+1</f>
         <v>46135</v>
       </c>
-      <c r="AV5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="CE5" s="22">
+        <f t="shared" ref="CE5" si="15">CD5+1</f>
         <v>46136</v>
       </c>
-      <c r="AW5" s="22">
-        <f t="shared" ca="1" si="0"/>
+      <c r="CF5" s="22">
+        <f t="shared" ref="CF5" si="16">CE5+1</f>
         <v>46137</v>
       </c>
-      <c r="AX5" s="23">
-        <f t="shared" ca="1" si="0"/>
+      <c r="CG5" s="22">
+        <f t="shared" ref="CG5" si="17">CF5+1</f>
         <v>46138</v>
       </c>
-      <c r="AY5" s="24">
-        <f ca="1">AX5+1</f>
+      <c r="CH5" s="24">
+        <f>CG5+1</f>
         <v>46139</v>
       </c>
-      <c r="AZ5" s="22">
-        <f ca="1">AY5+1</f>
+      <c r="CI5" s="22">
+        <f>CH5+1</f>
         <v>46140</v>
       </c>
-      <c r="BA5" s="22">
-        <f t="shared" ref="BA5:BE5" ca="1" si="1">AZ5+1</f>
+      <c r="CJ5" s="22">
+        <f t="shared" ref="CJ5" si="18">CI5+1</f>
         <v>46141</v>
       </c>
-      <c r="BB5" s="22">
-        <f t="shared" ca="1" si="1"/>
+      <c r="CK5" s="22">
+        <f t="shared" ref="CK5" si="19">CJ5+1</f>
         <v>46142</v>
       </c>
-      <c r="BC5" s="22">
-        <f t="shared" ca="1" si="1"/>
+      <c r="CL5" s="22">
+        <f t="shared" ref="CL5" si="20">CK5+1</f>
         <v>46143</v>
       </c>
-      <c r="BD5" s="22">
-        <f t="shared" ca="1" si="1"/>
+      <c r="CM5" s="22">
+        <f t="shared" ref="CM5" si="21">CL5+1</f>
         <v>46144</v>
       </c>
-      <c r="BE5" s="23">
-        <f t="shared" ca="1" si="1"/>
+      <c r="CN5" s="22">
+        <f t="shared" ref="CN5" si="22">CM5+1</f>
         <v>46145</v>
-      </c>
-      <c r="BF5" s="24">
-        <f ca="1">BE5+1</f>
-        <v>46146</v>
-      </c>
-      <c r="BG5" s="22">
-        <f ca="1">BF5+1</f>
-        <v>46147</v>
-      </c>
-      <c r="BH5" s="22">
-        <f t="shared" ref="BH5:BL5" ca="1" si="2">BG5+1</f>
-        <v>46148</v>
-      </c>
-      <c r="BI5" s="22">
-        <f t="shared" ca="1" si="2"/>
-        <v>46149</v>
-      </c>
-      <c r="BJ5" s="22">
-        <f t="shared" ca="1" si="2"/>
-        <v>46150</v>
-      </c>
-      <c r="BK5" s="22">
-        <f t="shared" ca="1" si="2"/>
-        <v>46151</v>
-      </c>
-      <c r="BL5" s="22">
-        <f t="shared" ca="1" si="2"/>
-        <v>46152</v>
-      </c>
-      <c r="BM5" s="24">
-        <f ca="1">BL5+1</f>
-        <v>46153</v>
-      </c>
-      <c r="BN5" s="22">
-        <f ca="1">BM5+1</f>
-        <v>46154</v>
-      </c>
-      <c r="BO5" s="22">
-        <f t="shared" ref="BO5" ca="1" si="3">BN5+1</f>
-        <v>46155</v>
-      </c>
-      <c r="BP5" s="22">
-        <f t="shared" ref="BP5" ca="1" si="4">BO5+1</f>
-        <v>46156</v>
-      </c>
-      <c r="BQ5" s="22">
-        <f t="shared" ref="BQ5" ca="1" si="5">BP5+1</f>
-        <v>46157</v>
-      </c>
-      <c r="BR5" s="22">
-        <f t="shared" ref="BR5" ca="1" si="6">BQ5+1</f>
-        <v>46158</v>
-      </c>
-      <c r="BS5" s="22">
-        <f t="shared" ref="BS5" ca="1" si="7">BR5+1</f>
-        <v>46159</v>
-      </c>
-      <c r="BT5" s="24">
-        <f ca="1">BS5+1</f>
-        <v>46160</v>
-      </c>
-      <c r="BU5" s="22">
-        <f ca="1">BT5+1</f>
-        <v>46161</v>
-      </c>
-      <c r="BV5" s="22">
-        <f t="shared" ref="BV5" ca="1" si="8">BU5+1</f>
-        <v>46162</v>
-      </c>
-      <c r="BW5" s="22">
-        <f t="shared" ref="BW5" ca="1" si="9">BV5+1</f>
-        <v>46163</v>
-      </c>
-      <c r="BX5" s="22">
-        <f t="shared" ref="BX5" ca="1" si="10">BW5+1</f>
-        <v>46164</v>
-      </c>
-      <c r="BY5" s="22">
-        <f t="shared" ref="BY5" ca="1" si="11">BX5+1</f>
-        <v>46165</v>
-      </c>
-      <c r="BZ5" s="22">
-        <f t="shared" ref="BZ5" ca="1" si="12">BY5+1</f>
-        <v>46166</v>
-      </c>
-      <c r="CA5" s="24">
-        <f ca="1">BZ5+1</f>
-        <v>46167</v>
-      </c>
-      <c r="CB5" s="22">
-        <f ca="1">CA5+1</f>
-        <v>46168</v>
-      </c>
-      <c r="CC5" s="22">
-        <f t="shared" ref="CC5" ca="1" si="13">CB5+1</f>
-        <v>46169</v>
-      </c>
-      <c r="CD5" s="22">
-        <f t="shared" ref="CD5" ca="1" si="14">CC5+1</f>
-        <v>46170</v>
-      </c>
-      <c r="CE5" s="22">
-        <f t="shared" ref="CE5" ca="1" si="15">CD5+1</f>
-        <v>46171</v>
-      </c>
-      <c r="CF5" s="22">
-        <f t="shared" ref="CF5" ca="1" si="16">CE5+1</f>
-        <v>46172</v>
-      </c>
-      <c r="CG5" s="22">
-        <f t="shared" ref="CG5" ca="1" si="17">CF5+1</f>
-        <v>46173</v>
-      </c>
-      <c r="CH5" s="24">
-        <f ca="1">CG5+1</f>
-        <v>46174</v>
-      </c>
-      <c r="CI5" s="22">
-        <f ca="1">CH5+1</f>
-        <v>46175</v>
-      </c>
-      <c r="CJ5" s="22">
-        <f t="shared" ref="CJ5" ca="1" si="18">CI5+1</f>
-        <v>46176</v>
-      </c>
-      <c r="CK5" s="22">
-        <f t="shared" ref="CK5" ca="1" si="19">CJ5+1</f>
-        <v>46177</v>
-      </c>
-      <c r="CL5" s="22">
-        <f t="shared" ref="CL5" ca="1" si="20">CK5+1</f>
-        <v>46178</v>
-      </c>
-      <c r="CM5" s="22">
-        <f t="shared" ref="CM5" ca="1" si="21">CL5+1</f>
-        <v>46179</v>
-      </c>
-      <c r="CN5" s="22">
-        <f t="shared" ref="CN5" ca="1" si="22">CM5+1</f>
-        <v>46180</v>
       </c>
     </row>
     <row r="6" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="119"/>
-      <c r="B6" s="121"/>
-      <c r="C6" s="123"/>
-      <c r="D6" s="123"/>
-      <c r="E6" s="126"/>
-      <c r="F6" s="126"/>
+      <c r="A6" s="113"/>
+      <c r="B6" s="115"/>
+      <c r="C6" s="117"/>
+      <c r="D6" s="117"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="112"/>
       <c r="I6" s="25" t="str">
-        <f t="shared" ref="I6:AN6" ca="1" si="23">LEFT(TEXT(I5,"ddd"),1)</f>
+        <f t="shared" ref="I6:AN6" si="23">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="J6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="K6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>W</v>
       </c>
       <c r="L6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="M6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>F</v>
       </c>
       <c r="N6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="O6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="P6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>M</v>
       </c>
       <c r="Q6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="R6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>W</v>
       </c>
       <c r="S6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="T6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>F</v>
       </c>
       <c r="U6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="V6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="W6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>M</v>
       </c>
       <c r="X6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="Y6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>W</v>
       </c>
       <c r="Z6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="AA6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>F</v>
       </c>
       <c r="AB6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="AC6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="AD6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>M</v>
       </c>
       <c r="AE6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="AF6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>W</v>
       </c>
       <c r="AG6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="AH6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>F</v>
       </c>
       <c r="AI6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="AJ6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>S</v>
       </c>
       <c r="AK6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>M</v>
       </c>
       <c r="AL6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="AM6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>W</v>
       </c>
       <c r="AN6" s="26" t="str">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" si="23"/>
         <v>T</v>
       </c>
       <c r="AO6" s="26" t="str">
-        <f t="shared" ref="AO6:BL6" ca="1" si="24">LEFT(TEXT(AO5,"ddd"),1)</f>
+        <f t="shared" ref="AO6:BL6" si="24">LEFT(TEXT(AO5,"ddd"),1)</f>
         <v>F</v>
       </c>
       <c r="AP6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="AQ6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="AR6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>M</v>
       </c>
       <c r="AS6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="AT6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>W</v>
       </c>
       <c r="AU6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="AV6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>F</v>
       </c>
       <c r="AW6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="AX6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="AY6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>M</v>
       </c>
       <c r="AZ6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="BA6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>W</v>
       </c>
       <c r="BB6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="BC6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>F</v>
       </c>
       <c r="BD6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="BE6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="BF6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>M</v>
       </c>
       <c r="BG6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="BH6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>W</v>
       </c>
       <c r="BI6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>T</v>
       </c>
       <c r="BJ6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>F</v>
       </c>
       <c r="BK6" s="26" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="BL6" s="27" t="str">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" si="24"/>
         <v>S</v>
       </c>
       <c r="BM6" s="26" t="str">
-        <f t="shared" ref="BM6:BS6" ca="1" si="25">LEFT(TEXT(BM5,"ddd"),1)</f>
+        <f t="shared" ref="BM6:BS6" si="25">LEFT(TEXT(BM5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="BN6" s="26" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>T</v>
       </c>
       <c r="BO6" s="26" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>W</v>
       </c>
       <c r="BP6" s="26" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>T</v>
       </c>
       <c r="BQ6" s="26" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>F</v>
       </c>
       <c r="BR6" s="26" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>S</v>
       </c>
       <c r="BS6" s="27" t="str">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" si="25"/>
         <v>S</v>
       </c>
       <c r="BT6" s="26" t="str">
-        <f t="shared" ref="BT6:BZ6" ca="1" si="26">LEFT(TEXT(BT5,"ddd"),1)</f>
+        <f t="shared" ref="BT6:BZ6" si="26">LEFT(TEXT(BT5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="BU6" s="26" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>T</v>
       </c>
       <c r="BV6" s="26" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>W</v>
       </c>
       <c r="BW6" s="26" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>T</v>
       </c>
       <c r="BX6" s="26" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>F</v>
       </c>
       <c r="BY6" s="26" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>S</v>
       </c>
       <c r="BZ6" s="27" t="str">
-        <f t="shared" ca="1" si="26"/>
+        <f t="shared" si="26"/>
         <v>S</v>
       </c>
       <c r="CA6" s="26" t="str">
-        <f t="shared" ref="CA6:CG6" ca="1" si="27">LEFT(TEXT(CA5,"ddd"),1)</f>
+        <f t="shared" ref="CA6:CG6" si="27">LEFT(TEXT(CA5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="CB6" s="26" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>T</v>
       </c>
       <c r="CC6" s="26" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>W</v>
       </c>
       <c r="CD6" s="26" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>T</v>
       </c>
       <c r="CE6" s="26" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>F</v>
       </c>
       <c r="CF6" s="26" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>S</v>
       </c>
       <c r="CG6" s="27" t="str">
-        <f t="shared" ca="1" si="27"/>
+        <f t="shared" si="27"/>
         <v>S</v>
       </c>
       <c r="CH6" s="26" t="str">
-        <f t="shared" ref="CH6:CN6" ca="1" si="28">LEFT(TEXT(CH5,"ddd"),1)</f>
+        <f t="shared" ref="CH6:CN6" si="28">LEFT(TEXT(CH5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="CI6" s="26" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>T</v>
       </c>
       <c r="CJ6" s="26" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>W</v>
       </c>
       <c r="CK6" s="26" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>T</v>
       </c>
       <c r="CL6" s="26" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>F</v>
       </c>
       <c r="CM6" s="26" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>S</v>
       </c>
       <c r="CN6" s="27" t="str">
-        <f t="shared" ca="1" si="28"/>
+        <f t="shared" si="28"/>
         <v>S</v>
       </c>
     </row>
@@ -3494,16 +3499,16 @@
         <v>0</v>
       </c>
       <c r="E9" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F9" s="92">
-        <f ca="1">E9+58</f>
+        <f>E9+58</f>
         <v>46122</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I9" s="39"/>
@@ -3601,16 +3606,16 @@
         <v>0</v>
       </c>
       <c r="E10" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F10" s="92">
-        <f ca="1">E10+58</f>
+        <f>E10+58</f>
         <v>46122</v>
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I10" s="39"/>
@@ -3708,16 +3713,16 @@
         <v>0</v>
       </c>
       <c r="E11" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F11" s="92">
-        <f ca="1">E11+58</f>
+        <f>E11+58</f>
         <v>46122</v>
       </c>
       <c r="G11" s="14"/>
       <c r="H11" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I11" s="39"/>
@@ -3815,16 +3820,16 @@
         <v>0</v>
       </c>
       <c r="E12" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F12" s="92">
-        <f ca="1">E12+58</f>
+        <f>E12+58</f>
         <v>46122</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I12" s="39"/>
@@ -3922,16 +3927,16 @@
         <v>0</v>
       </c>
       <c r="E13" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F13" s="92">
-        <f ca="1">E13+58</f>
+        <f>E13+58</f>
         <v>46122</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I13" s="39"/>
@@ -4029,16 +4034,16 @@
         <v>0</v>
       </c>
       <c r="E14" s="92">
-        <f ca="1">F13+1</f>
+        <f>F13+1</f>
         <v>46123</v>
       </c>
       <c r="F14" s="92">
-        <f ca="1">E14+7</f>
+        <f>E14+7</f>
         <v>46130</v>
       </c>
       <c r="G14" s="14"/>
       <c r="H14" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>8</v>
       </c>
       <c r="I14" s="39"/>
@@ -4235,16 +4240,16 @@
         <v>1</v>
       </c>
       <c r="E16" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F16" s="92">
-        <f ca="1">E16+58</f>
+        <f>E16+58</f>
         <v>46122</v>
       </c>
       <c r="G16" s="14"/>
       <c r="H16" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I16" s="39"/>
@@ -4342,16 +4347,16 @@
         <v>0</v>
       </c>
       <c r="E17" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F17" s="92">
-        <f ca="1">E17+58</f>
+        <f>E17+58</f>
         <v>46122</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I17" s="39"/>
@@ -4449,16 +4454,16 @@
         <v>0</v>
       </c>
       <c r="E18" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F18" s="93">
-        <f ca="1">F17</f>
+        <f>F17</f>
         <v>46122</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="4">
-        <f t="shared" ca="1" si="29"/>
+        <f t="shared" si="29"/>
         <v>59</v>
       </c>
       <c r="I18" s="39"/>
@@ -4655,16 +4660,16 @@
         <v>0.15</v>
       </c>
       <c r="E20" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F20" s="92">
-        <f ca="1">E20+58</f>
+        <f>E20+58</f>
         <v>46122</v>
       </c>
       <c r="G20" s="14"/>
       <c r="H20" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>59</v>
       </c>
       <c r="I20" s="39"/>
@@ -4760,11 +4765,11 @@
       <c r="C21" s="37"/>
       <c r="D21" s="38"/>
       <c r="E21" s="92">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F21" s="92">
-        <f ca="1">E21+58</f>
+        <f>E21+58</f>
         <v>46122</v>
       </c>
       <c r="G21" s="14"/>
@@ -4864,16 +4869,16 @@
         <v>0</v>
       </c>
       <c r="E22" s="92">
-        <f ca="1">F21+1</f>
+        <f>F21+1</f>
         <v>46123</v>
       </c>
       <c r="F22" s="93">
-        <f ca="1">E22+7</f>
+        <f>E22+7</f>
         <v>46130</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>8</v>
       </c>
       <c r="I22" s="39"/>
@@ -4986,16 +4991,16 @@
         <v>0.5</v>
       </c>
       <c r="E24" s="96">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F24" s="96">
-        <f ca="1">E24+20</f>
+        <f>E24+20</f>
         <v>46084</v>
       </c>
       <c r="G24" s="14"/>
       <c r="H24" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>21</v>
       </c>
       <c r="I24" s="39"/>
@@ -5093,16 +5098,16 @@
         <v>0.85</v>
       </c>
       <c r="E25" s="96">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F25" s="96">
-        <f ca="1">E25+9</f>
+        <f>E25+9</f>
         <v>46073</v>
       </c>
       <c r="G25" s="14"/>
       <c r="H25" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>10</v>
       </c>
       <c r="I25" s="39"/>
@@ -6151,16 +6156,16 @@
         <v>0.1</v>
       </c>
       <c r="E35" s="99">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F35" s="99">
-        <f ca="1">E35+14</f>
+        <f>E35+14</f>
         <v>46078</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>15</v>
       </c>
       <c r="I35" s="39"/>
@@ -6258,7 +6263,7 @@
         <v>0</v>
       </c>
       <c r="E36" s="99">
-        <f ca="1">F35+1</f>
+        <f>F35+1</f>
         <v>46079</v>
       </c>
       <c r="F36" s="99">
@@ -6267,7 +6272,7 @@
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>52</v>
       </c>
       <c r="I36" s="39"/>
@@ -6461,19 +6466,21 @@
       </c>
       <c r="C38" s="55"/>
       <c r="D38" s="56">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="E38" s="99">
-        <f ca="1">Project_Start</f>
+        <f>Project_Start</f>
         <v>46064</v>
       </c>
       <c r="F38" s="99">
-        <f ca="1">E38+21</f>
+        <f>E38+21</f>
         <v>46085</v>
       </c>
-      <c r="G38" s="14"/>
+      <c r="G38" s="128" t="s">
+        <v>65</v>
+      </c>
       <c r="H38" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>22</v>
       </c>
       <c r="I38" s="39"/>
@@ -6571,7 +6578,7 @@
         <v>0.3</v>
       </c>
       <c r="E39" s="99">
-        <f ca="1">F38</f>
+        <f>F38</f>
         <v>46085</v>
       </c>
       <c r="F39" s="99">
@@ -6580,7 +6587,7 @@
       </c>
       <c r="G39" s="14"/>
       <c r="H39" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>46</v>
       </c>
       <c r="I39" s="39"/>
@@ -6675,10 +6682,10 @@
       </c>
       <c r="C40" s="55"/>
       <c r="D40" s="56">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E40" s="99">
-        <f ca="1">F38</f>
+        <f>F38</f>
         <v>46085</v>
       </c>
       <c r="F40" s="99">
@@ -6982,7 +6989,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="102">
-        <f ca="1">E35</f>
+        <f>E35</f>
         <v>46064</v>
       </c>
       <c r="F43" s="102">
@@ -6991,7 +6998,7 @@
       </c>
       <c r="G43" s="14"/>
       <c r="H43" s="4">
-        <f t="shared" ca="1" si="30"/>
+        <f t="shared" si="30"/>
         <v>94</v>
       </c>
       <c r="I43" s="39"/>
@@ -7822,12 +7829,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="CH4:CN4"/>
     <mergeCell ref="Q2:Z2"/>
     <mergeCell ref="Q1:Z1"/>
@@ -7844,6 +7845,12 @@
     <mergeCell ref="BM4:BS4"/>
     <mergeCell ref="BT4:BZ4"/>
     <mergeCell ref="CA4:CG4"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D50">
     <cfRule type="dataBar" priority="102">
@@ -7864,7 +7871,7 @@
       <formula>AND(task_end&gt;=I$5,task_start&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I33:BK44 I4:BK8 I9:BZ10 BL14 I14:BK16 I19:BK21 I23:BK31 I32:BM32 BL33:BM33 BL36 BL40:BZ40 BL43:CA43 I47:BK48 BL44:BM44 I45:BM45">
+  <conditionalFormatting sqref="I33:BK44 I4:BK8 I9:BZ10 BL14 I14:BK16 I19:BK21 I23:BK31 I32:BM32 BL33:BM33 BL36 BL40:BZ40 BL43:CA43 BL44:BM44 I45:BM45 I47:BK48">
     <cfRule type="expression" dxfId="43" priority="80">
       <formula>AND(TODAY()&gt;=I$5, TODAY()&lt;J$5)</formula>
     </cfRule>
@@ -7914,7 +7921,7 @@
       <formula>AND(task_end&gt;=BL$5,task_start&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BL43:CA43 I43:BK44 I47:BK48 BL44:BM44 I45:BM45">
+  <conditionalFormatting sqref="BL43:CA43 I43:BK44 BL44:BM44 I45:BM45 I47:BK48">
     <cfRule type="expression" dxfId="33" priority="115">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
@@ -7942,7 +7949,7 @@
       <formula>AND(task_end&gt;=BM$5,task_start&lt;BN$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I46:BT46 BN44:BT45">
+  <conditionalFormatting sqref="BN44:BT45 I46:BT46">
     <cfRule type="expression" dxfId="27" priority="48">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
@@ -7955,7 +7962,7 @@
       <formula>AND(TODAY()&gt;=BL$5, TODAY()&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BS14:BT14 BM34:BR38 BM4:BR8 BM14:BR15 BM19:BR19 BM23:BR31 BN32:BS33 BM41:BR42 I46:BT46 BN44:BT45">
+  <conditionalFormatting sqref="BS14:BT14 BM34:BR38 BM4:BR8 BM14:BR15 BM19:BR19 BM23:BR31 BN32:BS33 BM41:BR42 BN44:BT45 I46:BT46">
     <cfRule type="expression" dxfId="24" priority="41">
       <formula>AND(TODAY()&gt;=I$5, TODAY()&lt;J$5)</formula>
     </cfRule>
@@ -7970,9 +7977,9 @@
       <formula>AND(task_end&gt;=BT$5,task_start&lt;BU$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BT37:BY38 BT4:BY8 BZ14 BT14:BY15 BT19:BY19 BT23:BY35 BT41:BY42 BU44:CA44 BM47:CA47">
+  <conditionalFormatting sqref="BT37:BY38 BT4:BY8 BZ14 BT14:BY15 BT19:BY19 BT23:BY35 BT41:BY42 BU44:CA44">
     <cfRule type="expression" dxfId="21" priority="32">
-      <formula>AND(TODAY()&gt;=BM$5, TODAY()&lt;BN$5)</formula>
+      <formula>AND(TODAY()&gt;=BT$5, TODAY()&lt;BU$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT38:BY38">
@@ -7985,12 +7992,12 @@
       <formula>AND(task_end&gt;=BT$5,task_start&lt;BU$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BU44:CA44 BM47:CA47">
+  <conditionalFormatting sqref="BU44:CA44">
     <cfRule type="expression" dxfId="18" priority="39">
-      <formula>AND(task_start&lt;=BM$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=BM$5)</formula>
+      <formula>AND(task_start&lt;=BU$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=BU$5)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="17" priority="40" stopIfTrue="1">
-      <formula>AND(task_end&gt;=BM$5,task_start&lt;BN$5)</formula>
+      <formula>AND(task_end&gt;=BU$5,task_start&lt;BV$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="CA9:CF10 I11:CF13 CA14:CF14 BM16:CF16 I17:CF18 CD20:CF21 I22:CF22">
@@ -8008,7 +8015,7 @@
       <formula>AND(task_end&gt;=BL$5,task_start&lt;BM$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="CA37:CF38 CA4:CF10 I11:CF13 CA14:CF15 BL16:CF16 I17:CF18 CA19:CF19 BL20:CF21 I22:CF22 CA23:CF32 BZ33:CF33 CA34:CF35 BS36:CF36 BL39:CF39 CA40:CF42 CB43:CF44 BU45:CF46 CB47:CF47">
+  <conditionalFormatting sqref="CA37:CF38 CA4:CF10 I11:CF13 CA14:CF15 BL16:CF16 I17:CF18 CA19:CF19 BL20:CF21 I22:CF22 CA23:CF32 BZ33:CF33 CA34:CF35 BS36:CF36 BL39:CF39 CA40:CF42 CB43:CF44 BU45:CF46 BM47:CF47">
     <cfRule type="expression" dxfId="13" priority="23">
       <formula>AND(TODAY()&gt;=I$5, TODAY()&lt;J$5)</formula>
     </cfRule>
@@ -8018,12 +8025,12 @@
       <formula>AND(task_end&gt;=CA$5,task_start&lt;CB$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="CB43:CF44 BU45:CF46 CB47:CF47">
+  <conditionalFormatting sqref="CB43:CF44 BU45:CF46 BM47:CF47">
     <cfRule type="expression" dxfId="11" priority="30">
-      <formula>AND(task_start&lt;=BU$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=BU$5)</formula>
+      <formula>AND(task_start&lt;=BM$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=BM$5)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="10" priority="31" stopIfTrue="1">
-      <formula>AND(task_end&gt;=BU$5,task_start&lt;BV$5)</formula>
+      <formula>AND(task_end&gt;=BM$5,task_start&lt;BN$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="CG9:CG14 CN9:CN14 BS14 CG16:CG18 CN16:CN18 CG20:CG22 CN20:CN22">
@@ -8274,6 +8281,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -8585,36 +8621,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2348D59-3426-404A-A0C5-6456F6613EDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8635,26 +8662,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
Finished testing  - testing (besides cost)
</commit_message>
<xml_diff>
--- a/resources/TierPlus Planning.xlsx
+++ b/resources/TierPlus Planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="538" documentId="8_{E97B7BBA-A1CF-CA4D-89B6-D5BE4B7D4A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC8E3A57-2325-104B-BBE7-A1E78C60678F}"/>
+  <xr:revisionPtr revIDLastSave="539" documentId="8_{E97B7BBA-A1CF-CA4D-89B6-D5BE4B7D4A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F97C446-34F2-1F42-AA24-11415B47F62C}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5100,7 +5100,7 @@
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="49">
-        <v>0.85</v>
+        <v>100</v>
       </c>
       <c r="E25" s="96">
         <f>Project_Start</f>

</xml_diff>

<commit_message>
SOuth Africa mortality calibration only
</commit_message>
<xml_diff>
--- a/resources/TierPlus Planning.xlsx
+++ b/resources/TierPlus Planning.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -48,6 +48,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="67">
   <si>
+    <t>Tier Plus</t>
+  </si>
+  <si>
     <t>Project start:</t>
   </si>
   <si>
@@ -57,7 +60,7 @@
     <t>Display week:</t>
   </si>
   <si>
-    <t>SIMPLE GANTT CHART by Vertex42.com</t>
+    <t>scroll to see more dates</t>
   </si>
   <si>
     <t>https://www.vertex42.com/ExcelTemplates/simple-gantt-chart.html</t>
@@ -81,7 +84,130 @@
     <t xml:space="preserve">Do not delete this row. This row is hidden to preserve a formula that is used to highlight the current day within the project schedule. </t>
   </si>
   <si>
+    <t>Data Collection - Efficacy and Cost params</t>
+  </si>
+  <si>
+    <t>Prevention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing </t>
+  </si>
+  <si>
+    <t>Monitoring and retention</t>
+  </si>
+  <si>
+    <t>AHD and prophylaxis</t>
+  </si>
+  <si>
+    <t>ANC and PNC</t>
+  </si>
+  <si>
+    <t>Costing</t>
+  </si>
+  <si>
+    <t>Test app integration</t>
+  </si>
+  <si>
+    <t>Data Collection - Additional assumption and rates (e.g mortality rates per group)</t>
+  </si>
+  <si>
+    <t>Create parameter list with dummy values</t>
+  </si>
+  <si>
+    <t>Collect data</t>
+  </si>
+  <si>
+    <t>Integrate into app</t>
+  </si>
+  <si>
+    <t>Data Collection - Baseline intervention values (where available)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collect any available data </t>
+  </si>
+  <si>
+    <t>Define assumptions for baseline interventions in the abscence of data</t>
+  </si>
+  <si>
+    <t>Integrate both into app</t>
+  </si>
+  <si>
+    <t>Core Logic Testing - test code and documentation - usually results in app fixes as well</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Mortality</t>
+  </si>
+  <si>
+    <t>General viral suppression and infections</t>
+  </si>
+  <si>
+    <t>Populations and 95's (potentially incoporated in during above sections)</t>
+  </si>
+  <si>
+    <t>Relative scenario and baseline counts</t>
+  </si>
+  <si>
+    <t>Re-test with all new data</t>
+  </si>
+  <si>
+    <t>Validation - Logic (some incoporated during core logic testing)</t>
+  </si>
+  <si>
+    <t>Define validation cases, logic and assumptions (including eligble populations, minimum or maximum groups, overlapping interventions, impact on 90's etc)</t>
+  </si>
+  <si>
+    <t>Implement and Test</t>
+  </si>
+  <si>
+    <t>Input Validation - App - Implement and test</t>
+  </si>
+  <si>
+    <t>Define validation cases, logic and assumption (e.g prep_len + prep_oral cannot exceed eligible pop)</t>
+  </si>
+  <si>
+    <t>Need a check for if I'm missing things</t>
+  </si>
+  <si>
+    <t>Implement: Input limits (where relevant)</t>
+  </si>
+  <si>
+    <t>Implement: Limits on combinations (prep+mmd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement: </t>
+  </si>
+  <si>
+    <t>Integrated Testing and User feedback</t>
+  </si>
+  <si>
+    <t>Figure out app publishing</t>
+  </si>
+  <si>
+    <t>Test reasonable scenarios</t>
+  </si>
+  <si>
+    <t>Test unreasonable scenarios</t>
+  </si>
+  <si>
+    <t>Fix problems</t>
+  </si>
+  <si>
+    <t>Gather user feedback</t>
+  </si>
+  <si>
+    <t>Integrate feedback</t>
+  </si>
+  <si>
+    <t>END PLANNING: JUNE 15th Max</t>
+  </si>
+  <si>
     <t>Insert new rows ABOVE this one</t>
+  </si>
+  <si>
+    <t>SIMPLE GANTT CHART by Vertex42.com</t>
   </si>
   <si>
     <t>About This Template</t>
@@ -127,132 +253,6 @@
   <si>
     <t>Businesses will find invoices, time sheets, inventory trackers, financial statements, and project planning templates. Teachers and students will find resources such as class schedules, grade books, and attendance sheets. Organize your family life with meal planners, checklists, and exercise logs. Each template is thoroughly researched, refined, and improved over time through feedback from thousands of users.</t>
   </si>
-  <si>
-    <t>Tier Plus</t>
-  </si>
-  <si>
-    <t>Data Collection - Efficacy and Cost params</t>
-  </si>
-  <si>
-    <t>Prevention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing </t>
-  </si>
-  <si>
-    <t>Monitoring and retention</t>
-  </si>
-  <si>
-    <t>AHD and prophylaxis</t>
-  </si>
-  <si>
-    <t>ANC and PNC</t>
-  </si>
-  <si>
-    <t>Data Collection - Additional assumption and rates (e.g mortality rates per group)</t>
-  </si>
-  <si>
-    <t>Collect data</t>
-  </si>
-  <si>
-    <t>Integrate into app</t>
-  </si>
-  <si>
-    <t>Create parameter list with dummy values</t>
-  </si>
-  <si>
-    <t>Data Collection - Baseline intervention values (where available)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collect any available data </t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>General viral suppression and infections</t>
-  </si>
-  <si>
-    <t>Costing</t>
-  </si>
-  <si>
-    <t>Test app integration</t>
-  </si>
-  <si>
-    <t>Implement and Test</t>
-  </si>
-  <si>
-    <t>Define validation cases, logic and assumptions (including eligble populations, minimum or maximum groups, overlapping interventions, impact on 90's etc)</t>
-  </si>
-  <si>
-    <t>Input Validation - App - Implement and test</t>
-  </si>
-  <si>
-    <t>Define validation cases, logic and assumption (e.g prep_len + prep_oral cannot exceed eligible pop)</t>
-  </si>
-  <si>
-    <t>Integrated Testing and User feedback</t>
-  </si>
-  <si>
-    <t>Test unreasonable scenarios</t>
-  </si>
-  <si>
-    <t>Fix problems</t>
-  </si>
-  <si>
-    <t>Gather user feedback</t>
-  </si>
-  <si>
-    <t>Integrate feedback</t>
-  </si>
-  <si>
-    <t>Test reasonable scenarios</t>
-  </si>
-  <si>
-    <t>Integrate both into app</t>
-  </si>
-  <si>
-    <t>Core Logic Testing - test code and documentation - usually results in app fixes as well</t>
-  </si>
-  <si>
-    <t>Populations and 95's (potentially incoporated in during above sections)</t>
-  </si>
-  <si>
-    <t>Implement: Input limits (where relevant)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement: </t>
-  </si>
-  <si>
-    <t>END PLANNING: JUNE 15th Max</t>
-  </si>
-  <si>
-    <t>Figure out app publishing</t>
-  </si>
-  <si>
-    <t>Validation - Logic (some incoporated during core logic testing)</t>
-  </si>
-  <si>
-    <t>Re-test with all new data</t>
-  </si>
-  <si>
-    <t>Mortality</t>
-  </si>
-  <si>
-    <t>scroll to see more dates</t>
-  </si>
-  <si>
-    <t>Define assumptions for baseline interventions in the abscence of data</t>
-  </si>
-  <si>
-    <t>Need a check for if I'm missing things</t>
-  </si>
-  <si>
-    <t>Implement: Limits on combinations (prep+mmd)</t>
-  </si>
-  <si>
-    <t>Relative scenario and baseline counts</t>
-  </si>
 </sst>
 </file>
 
@@ -267,7 +267,7 @@
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="169" formatCode="[$-409]d\-mmm;@"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -849,7 +849,7 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1069,9 +1069,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1154,6 +1151,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="19" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1163,38 +1182,20 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="27" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="19" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="20" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="4" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Comma" xfId="4" builtinId="3" customBuiltin="1"/>
@@ -1205,7 +1206,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Name" xfId="11" xr:uid="{B2D3C1EE-6B41-4801-AAFC-C2274E49E503}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
     <cellStyle name="Project Start" xfId="9" xr:uid="{8EB8A09A-C31C-40A3-B2C1-9449520178B8}"/>
     <cellStyle name="Task" xfId="12" xr:uid="{6391D789-272B-4DD2-9BF3-2CDCF610FA41}"/>
     <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
@@ -2378,238 +2379,331 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:CN55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" style="12" customWidth="1"/>
-    <col min="2" max="2" width="37.33203125" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" style="106" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" style="107" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.83203125" customWidth="1"/>
-    <col min="8" max="8" width="0.6640625" customWidth="1"/>
-    <col min="9" max="92" width="2.6640625" customWidth="1"/>
+    <col min="1" max="1" width="2.625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="37.375" customWidth="1"/>
+    <col min="3" max="3" width="16.625" customWidth="1"/>
+    <col min="4" max="4" width="10.625" customWidth="1"/>
+    <col min="5" max="5" width="10.625" style="105" customWidth="1"/>
+    <col min="6" max="6" width="6.625" style="106" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.875" customWidth="1"/>
+    <col min="8" max="8" width="0.625" customWidth="1"/>
+    <col min="9" max="92" width="2.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:92" ht="90" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="A1" s="81"/>
+    <row r="1" spans="1:92" ht="90" customHeight="1">
+      <c r="A1" s="112"/>
       <c r="B1" s="73" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C1" s="15"/>
       <c r="D1" s="16"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="83"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="82"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
+      <c r="I1" s="123" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="125"/>
+      <c r="K1" s="125"/>
+      <c r="L1" s="125"/>
+      <c r="M1" s="125"/>
+      <c r="N1" s="125"/>
+      <c r="O1" s="125"/>
       <c r="P1" s="18"/>
-      <c r="Q1" s="116">
+      <c r="Q1" s="122">
         <v>46064</v>
       </c>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
+      <c r="R1" s="126"/>
+      <c r="S1" s="126"/>
+      <c r="T1" s="126"/>
+      <c r="U1" s="126"/>
+      <c r="V1" s="126"/>
+      <c r="W1" s="126"/>
+      <c r="X1" s="126"/>
+      <c r="Y1" s="126"/>
+      <c r="Z1" s="126"/>
     </row>
-    <row r="2" spans="1:92" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:92" ht="30" customHeight="1">
       <c r="B2" s="71"/>
       <c r="C2" s="72" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="17"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="85"/>
-      <c r="I2" s="118" t="s">
-        <v>2</v>
-      </c>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="84"/>
+      <c r="I2" s="123" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="125"/>
+      <c r="K2" s="125"/>
+      <c r="L2" s="125"/>
+      <c r="M2" s="125"/>
+      <c r="N2" s="125"/>
+      <c r="O2" s="125"/>
       <c r="P2" s="18"/>
-      <c r="Q2" s="114">
+      <c r="Q2" s="121">
         <v>5</v>
       </c>
-      <c r="R2" s="115"/>
-      <c r="S2" s="115"/>
-      <c r="T2" s="115"/>
-      <c r="U2" s="115"/>
-      <c r="V2" s="115"/>
-      <c r="W2" s="115"/>
-      <c r="X2" s="115"/>
-      <c r="Y2" s="115"/>
-      <c r="Z2" s="115"/>
+      <c r="R2" s="127"/>
+      <c r="S2" s="127"/>
+      <c r="T2" s="127"/>
+      <c r="U2" s="127"/>
+      <c r="V2" s="127"/>
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
+      <c r="Z2" s="127"/>
       <c r="AP2" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:92" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:92" s="20" customFormat="1" ht="30" customHeight="1">
       <c r="A3" s="12"/>
       <c r="B3" s="19"/>
+      <c r="C3" s="111"/>
       <c r="D3" s="21"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="87"/>
+      <c r="E3" s="85"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
+      <c r="M3" s="111"/>
+      <c r="N3" s="111"/>
+      <c r="O3" s="111"/>
+      <c r="P3" s="111"/>
+      <c r="Q3" s="111"/>
+      <c r="R3" s="111"/>
+      <c r="S3" s="111"/>
+      <c r="T3" s="111"/>
+      <c r="U3" s="111"/>
+      <c r="V3" s="111"/>
+      <c r="W3" s="111"/>
+      <c r="X3" s="111"/>
+      <c r="Y3" s="111"/>
+      <c r="Z3" s="111"/>
+      <c r="AA3" s="111"/>
+      <c r="AB3" s="111"/>
+      <c r="AC3" s="111"/>
+      <c r="AD3" s="111"/>
+      <c r="AE3" s="111"/>
+      <c r="AF3" s="111"/>
+      <c r="AG3" s="111"/>
+      <c r="AH3" s="111"/>
+      <c r="AI3" s="111"/>
+      <c r="AJ3" s="111"/>
+      <c r="AK3" s="111"/>
+      <c r="AL3" s="111"/>
+      <c r="AM3" s="111"/>
+      <c r="AN3" s="111"/>
+      <c r="AO3" s="111"/>
+      <c r="AP3" s="111"/>
+      <c r="AQ3" s="111"/>
+      <c r="AR3" s="111"/>
+      <c r="AS3" s="111"/>
+      <c r="AT3" s="111"/>
+      <c r="AU3" s="111"/>
+      <c r="AV3" s="111"/>
+      <c r="AW3" s="111"/>
+      <c r="AX3" s="111"/>
+      <c r="AY3" s="111"/>
+      <c r="AZ3" s="111"/>
+      <c r="BA3" s="111"/>
+      <c r="BB3" s="111"/>
+      <c r="BC3" s="111"/>
+      <c r="BD3" s="111"/>
+      <c r="BE3" s="111"/>
+      <c r="BF3" s="111"/>
+      <c r="BG3" s="111"/>
+      <c r="BH3" s="111"/>
+      <c r="BI3" s="111"/>
+      <c r="BJ3" s="111"/>
+      <c r="BK3" s="111"/>
+      <c r="BL3" s="111"/>
+      <c r="BM3" s="111"/>
+      <c r="BN3" s="111"/>
+      <c r="BO3" s="111"/>
+      <c r="BP3" s="111"/>
+      <c r="BQ3" s="111"/>
+      <c r="BR3" s="111"/>
+      <c r="BS3" s="111"/>
+      <c r="BT3" s="111"/>
+      <c r="BU3" s="111"/>
+      <c r="BV3" s="111"/>
+      <c r="BW3" s="111"/>
+      <c r="BX3" s="111"/>
+      <c r="BY3" s="111"/>
+      <c r="BZ3" s="111"/>
+      <c r="CA3" s="111"/>
+      <c r="CB3" s="111"/>
+      <c r="CC3" s="111"/>
+      <c r="CD3" s="111"/>
+      <c r="CE3" s="111"/>
+      <c r="CF3" s="111"/>
+      <c r="CG3" s="111"/>
+      <c r="CH3" s="111"/>
+      <c r="CI3" s="111"/>
+      <c r="CJ3" s="111"/>
+      <c r="CK3" s="111"/>
+      <c r="CL3" s="111"/>
+      <c r="CM3" s="111"/>
+      <c r="CN3" s="111"/>
     </row>
-    <row r="4" spans="1:92" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="81"/>
-      <c r="B4" s="110" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="88"/>
-      <c r="F4" s="87"/>
-      <c r="I4" s="120">
+    <row r="4" spans="1:92" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A4" s="112"/>
+      <c r="B4" s="109" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="111"/>
+      <c r="D4" s="111"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="124">
         <f>I5</f>
         <v>46090</v>
       </c>
-      <c r="J4" s="112"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="112"/>
-      <c r="M4" s="112"/>
-      <c r="N4" s="112"/>
-      <c r="O4" s="112"/>
-      <c r="P4" s="112">
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="119">
         <f>P5</f>
         <v>46097</v>
       </c>
-      <c r="Q4" s="112"/>
-      <c r="R4" s="112"/>
-      <c r="S4" s="112"/>
-      <c r="T4" s="112"/>
-      <c r="U4" s="112"/>
-      <c r="V4" s="112"/>
-      <c r="W4" s="112">
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
+      <c r="U4" s="119"/>
+      <c r="V4" s="119"/>
+      <c r="W4" s="119">
         <f>W5</f>
         <v>46104</v>
       </c>
-      <c r="X4" s="112"/>
-      <c r="Y4" s="112"/>
-      <c r="Z4" s="112"/>
-      <c r="AA4" s="112"/>
-      <c r="AB4" s="112"/>
-      <c r="AC4" s="112"/>
-      <c r="AD4" s="112">
+      <c r="X4" s="119"/>
+      <c r="Y4" s="119"/>
+      <c r="Z4" s="119"/>
+      <c r="AA4" s="119"/>
+      <c r="AB4" s="119"/>
+      <c r="AC4" s="119"/>
+      <c r="AD4" s="119">
         <f>AD5</f>
         <v>46111</v>
       </c>
-      <c r="AE4" s="112"/>
-      <c r="AF4" s="112"/>
-      <c r="AG4" s="112"/>
-      <c r="AH4" s="112"/>
-      <c r="AI4" s="112"/>
-      <c r="AJ4" s="112"/>
-      <c r="AK4" s="112">
+      <c r="AE4" s="119"/>
+      <c r="AF4" s="119"/>
+      <c r="AG4" s="119"/>
+      <c r="AH4" s="119"/>
+      <c r="AI4" s="119"/>
+      <c r="AJ4" s="119"/>
+      <c r="AK4" s="119">
         <f>AK5</f>
         <v>46118</v>
       </c>
-      <c r="AL4" s="112"/>
-      <c r="AM4" s="112"/>
-      <c r="AN4" s="112"/>
-      <c r="AO4" s="112"/>
-      <c r="AP4" s="112"/>
-      <c r="AQ4" s="112"/>
-      <c r="AR4" s="112">
+      <c r="AL4" s="119"/>
+      <c r="AM4" s="119"/>
+      <c r="AN4" s="119"/>
+      <c r="AO4" s="119"/>
+      <c r="AP4" s="119"/>
+      <c r="AQ4" s="119"/>
+      <c r="AR4" s="119">
         <f>AR5</f>
         <v>46125</v>
       </c>
-      <c r="AS4" s="112"/>
-      <c r="AT4" s="112"/>
-      <c r="AU4" s="112"/>
-      <c r="AV4" s="112"/>
-      <c r="AW4" s="112"/>
-      <c r="AX4" s="112"/>
-      <c r="AY4" s="112">
+      <c r="AS4" s="119"/>
+      <c r="AT4" s="119"/>
+      <c r="AU4" s="119"/>
+      <c r="AV4" s="119"/>
+      <c r="AW4" s="119"/>
+      <c r="AX4" s="119"/>
+      <c r="AY4" s="119">
         <f>AY5</f>
         <v>46132</v>
       </c>
-      <c r="AZ4" s="112"/>
-      <c r="BA4" s="112"/>
-      <c r="BB4" s="112"/>
-      <c r="BC4" s="112"/>
-      <c r="BD4" s="112"/>
-      <c r="BE4" s="112"/>
-      <c r="BF4" s="112">
+      <c r="AZ4" s="119"/>
+      <c r="BA4" s="119"/>
+      <c r="BB4" s="119"/>
+      <c r="BC4" s="119"/>
+      <c r="BD4" s="119"/>
+      <c r="BE4" s="119"/>
+      <c r="BF4" s="119">
         <f>BF5</f>
         <v>46139</v>
       </c>
-      <c r="BG4" s="112"/>
-      <c r="BH4" s="112"/>
-      <c r="BI4" s="112"/>
-      <c r="BJ4" s="112"/>
-      <c r="BK4" s="112"/>
-      <c r="BL4" s="113"/>
-      <c r="BM4" s="112">
+      <c r="BG4" s="119"/>
+      <c r="BH4" s="119"/>
+      <c r="BI4" s="119"/>
+      <c r="BJ4" s="119"/>
+      <c r="BK4" s="119"/>
+      <c r="BL4" s="120"/>
+      <c r="BM4" s="119">
         <f>BM5</f>
         <v>46146</v>
       </c>
-      <c r="BN4" s="112"/>
-      <c r="BO4" s="112"/>
-      <c r="BP4" s="112"/>
-      <c r="BQ4" s="112"/>
-      <c r="BR4" s="112"/>
-      <c r="BS4" s="113"/>
-      <c r="BT4" s="112">
+      <c r="BN4" s="119"/>
+      <c r="BO4" s="119"/>
+      <c r="BP4" s="119"/>
+      <c r="BQ4" s="119"/>
+      <c r="BR4" s="119"/>
+      <c r="BS4" s="120"/>
+      <c r="BT4" s="119">
         <f>BT5</f>
         <v>46153</v>
       </c>
-      <c r="BU4" s="112"/>
-      <c r="BV4" s="112"/>
-      <c r="BW4" s="112"/>
-      <c r="BX4" s="112"/>
-      <c r="BY4" s="112"/>
-      <c r="BZ4" s="113"/>
-      <c r="CA4" s="112">
+      <c r="BU4" s="119"/>
+      <c r="BV4" s="119"/>
+      <c r="BW4" s="119"/>
+      <c r="BX4" s="119"/>
+      <c r="BY4" s="119"/>
+      <c r="BZ4" s="120"/>
+      <c r="CA4" s="119">
         <f>CA5</f>
         <v>46160</v>
       </c>
-      <c r="CB4" s="112"/>
-      <c r="CC4" s="112"/>
-      <c r="CD4" s="112"/>
-      <c r="CE4" s="112"/>
-      <c r="CF4" s="112"/>
-      <c r="CG4" s="113"/>
-      <c r="CH4" s="112">
+      <c r="CB4" s="119"/>
+      <c r="CC4" s="119"/>
+      <c r="CD4" s="119"/>
+      <c r="CE4" s="119"/>
+      <c r="CF4" s="119"/>
+      <c r="CG4" s="120"/>
+      <c r="CH4" s="119">
         <f>CH5</f>
         <v>46167</v>
       </c>
-      <c r="CI4" s="112"/>
-      <c r="CJ4" s="112"/>
-      <c r="CK4" s="112"/>
-      <c r="CL4" s="112"/>
-      <c r="CM4" s="112"/>
-      <c r="CN4" s="113"/>
+      <c r="CI4" s="119"/>
+      <c r="CJ4" s="119"/>
+      <c r="CK4" s="119"/>
+      <c r="CL4" s="119"/>
+      <c r="CM4" s="119"/>
+      <c r="CN4" s="120"/>
     </row>
-    <row r="5" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="123"/>
-      <c r="B5" s="124" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="126" t="s">
+    <row r="5" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1">
+      <c r="A5" s="114"/>
+      <c r="B5" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="128" t="s">
+      <c r="C5" s="117" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="121" t="s">
+      <c r="D5" s="118" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="121" t="s">
+      <c r="E5" s="113" t="s">
         <v>9</v>
       </c>
+      <c r="F5" s="113" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="111"/>
+      <c r="H5" s="111"/>
       <c r="I5" s="22">
         <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
         <v>46090</v>
@@ -2947,13 +3041,15 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="6" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="123"/>
-      <c r="B6" s="125"/>
-      <c r="C6" s="127"/>
-      <c r="D6" s="127"/>
-      <c r="E6" s="122"/>
-      <c r="F6" s="122"/>
+    <row r="6" spans="1:92" s="20" customFormat="1" ht="15" customHeight="1" thickBot="1">
+      <c r="A6" s="114"/>
+      <c r="B6" s="116"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="128"/>
+      <c r="E6" s="129"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
       <c r="I6" s="25" t="str">
         <f t="shared" ref="I6:AN6" si="23">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>M</v>
@@ -3291,17 +3387,18 @@
         <v>S</v>
       </c>
     </row>
-    <row r="7" spans="1:92" s="20" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:92" s="20" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1">
       <c r="A7" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="29"/>
       <c r="D7" s="28"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="89"/>
-      <c r="H7" s="20" t="str">
-        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="E7" s="88"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111" t="str">
+        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I7" s="30"/>
@@ -3389,18 +3486,18 @@
       <c r="CM7" s="30"/>
       <c r="CN7" s="30"/>
     </row>
-    <row r="8" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="81"/>
+    <row r="8" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A8" s="112"/>
       <c r="B8" s="31" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C8" s="32"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="90"/>
-      <c r="F8" s="91"/>
+      <c r="E8" s="89"/>
+      <c r="F8" s="90"/>
       <c r="G8" s="14"/>
       <c r="H8" s="4" t="str">
-        <f t="shared" ref="H8:H19" si="29">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H8:H19" ca="1" si="29">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="34"/>
@@ -3488,26 +3585,26 @@
       <c r="CM8" s="34"/>
       <c r="CN8" s="34"/>
     </row>
-    <row r="9" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="81"/>
+    <row r="9" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A9" s="112"/>
       <c r="B9" s="36" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="38">
         <v>0</v>
       </c>
-      <c r="E9" s="92">
+      <c r="E9" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F9" s="92">
+      <c r="F9" s="91">
         <f>E9+58</f>
         <v>46122</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I9" s="39"/>
@@ -3595,26 +3692,26 @@
       <c r="CM9" s="39"/>
       <c r="CN9" s="39"/>
     </row>
-    <row r="10" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="81"/>
+    <row r="10" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A10" s="112"/>
       <c r="B10" s="40" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C10" s="41"/>
       <c r="D10" s="42">
         <v>0.8</v>
       </c>
-      <c r="E10" s="92">
+      <c r="E10" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F10" s="92">
+      <c r="F10" s="91">
         <f>E10+58</f>
         <v>46122</v>
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I10" s="39"/>
@@ -3702,26 +3799,26 @@
       <c r="CM10" s="39"/>
       <c r="CN10" s="39"/>
     </row>
-    <row r="11" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A11" s="12"/>
       <c r="B11" s="40" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C11" s="41"/>
       <c r="D11" s="42">
         <v>0</v>
       </c>
-      <c r="E11" s="92">
+      <c r="E11" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F11" s="92">
+      <c r="F11" s="91">
         <f>E11+58</f>
         <v>46122</v>
       </c>
       <c r="G11" s="14"/>
       <c r="H11" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I11" s="39"/>
@@ -3809,26 +3906,26 @@
       <c r="CM11" s="39"/>
       <c r="CN11" s="39"/>
     </row>
-    <row r="12" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A12" s="12"/>
       <c r="B12" s="40" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C12" s="41"/>
       <c r="D12" s="42">
         <v>0</v>
       </c>
-      <c r="E12" s="92">
+      <c r="E12" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F12" s="92">
+      <c r="F12" s="91">
         <f>E12+58</f>
         <v>46122</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I12" s="39"/>
@@ -3916,26 +4013,26 @@
       <c r="CM12" s="39"/>
       <c r="CN12" s="39"/>
     </row>
-    <row r="13" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A13" s="12"/>
       <c r="B13" s="40" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C13" s="41"/>
       <c r="D13" s="42">
         <v>0</v>
       </c>
-      <c r="E13" s="92">
+      <c r="E13" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F13" s="92">
+      <c r="F13" s="91">
         <f>E13+58</f>
         <v>46122</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I13" s="39"/>
@@ -4023,20 +4120,20 @@
       <c r="CM13" s="39"/>
       <c r="CN13" s="39"/>
     </row>
-    <row r="14" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A14" s="12"/>
       <c r="B14" s="40" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C14" s="41"/>
       <c r="D14" s="42">
         <v>0.9</v>
       </c>
-      <c r="E14" s="92">
+      <c r="E14" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F14" s="92">
+      <c r="F14" s="91">
         <f>E14+58</f>
         <v>46122</v>
       </c>
@@ -4127,26 +4224,26 @@
       <c r="CM14" s="39"/>
       <c r="CN14" s="39"/>
     </row>
-    <row r="15" spans="1:92" s="35" customFormat="1" ht="53" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:92" s="35" customFormat="1" ht="53.1" customHeight="1" thickBot="1">
       <c r="A15" s="12"/>
       <c r="B15" s="40" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="C15" s="41"/>
       <c r="D15" s="42">
         <v>0</v>
       </c>
-      <c r="E15" s="92">
+      <c r="E15" s="91">
         <f>F13+1</f>
         <v>46123</v>
       </c>
-      <c r="F15" s="92">
+      <c r="F15" s="91">
         <f>E15+14</f>
         <v>46137</v>
       </c>
-      <c r="G15" s="111"/>
+      <c r="G15" s="110"/>
       <c r="H15" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>15</v>
       </c>
       <c r="I15" s="39"/>
@@ -4234,18 +4331,18 @@
       <c r="CM15" s="39"/>
       <c r="CN15" s="39"/>
     </row>
-    <row r="16" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="81"/>
+    <row r="16" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A16" s="112"/>
       <c r="B16" s="31" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C16" s="32"/>
       <c r="D16" s="33"/>
-      <c r="E16" s="90"/>
-      <c r="F16" s="91"/>
+      <c r="E16" s="89"/>
+      <c r="F16" s="90"/>
       <c r="G16" s="14"/>
       <c r="H16" s="4" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v/>
       </c>
       <c r="I16" s="34"/>
@@ -4333,26 +4430,26 @@
       <c r="CM16" s="34"/>
       <c r="CN16" s="34"/>
     </row>
-    <row r="17" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="81"/>
+    <row r="17" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A17" s="112"/>
       <c r="B17" s="36" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C17" s="37"/>
       <c r="D17" s="38">
         <v>1</v>
       </c>
-      <c r="E17" s="92">
+      <c r="E17" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F17" s="92">
+      <c r="F17" s="91">
         <f>E17+58</f>
         <v>46122</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I17" s="39"/>
@@ -4440,26 +4537,26 @@
       <c r="CM17" s="39"/>
       <c r="CN17" s="39"/>
     </row>
-    <row r="18" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="81"/>
+    <row r="18" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A18" s="112"/>
       <c r="B18" s="40" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C18" s="41"/>
       <c r="D18" s="42">
         <v>0</v>
       </c>
-      <c r="E18" s="92">
+      <c r="E18" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F18" s="92">
+      <c r="F18" s="91">
         <f>E18+58</f>
         <v>46122</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I18" s="39"/>
@@ -4547,26 +4644,26 @@
       <c r="CM18" s="39"/>
       <c r="CN18" s="39"/>
     </row>
-    <row r="19" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A19" s="12"/>
       <c r="B19" s="40" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="C19" s="41"/>
       <c r="D19" s="42">
         <v>0</v>
       </c>
-      <c r="E19" s="92">
+      <c r="E19" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F19" s="93">
+      <c r="F19" s="92">
         <f>F18</f>
         <v>46122</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="4">
-        <f t="shared" si="29"/>
+        <f t="shared" ca="1" si="29"/>
         <v>59</v>
       </c>
       <c r="I19" s="39"/>
@@ -4654,18 +4751,18 @@
       <c r="CM19" s="39"/>
       <c r="CN19" s="39"/>
     </row>
-    <row r="20" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="81"/>
+    <row r="20" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A20" s="112"/>
       <c r="B20" s="31" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="33"/>
-      <c r="E20" s="90"/>
-      <c r="F20" s="91"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="90"/>
       <c r="G20" s="14"/>
       <c r="H20" s="4" t="str">
-        <f t="shared" ref="H20:H52" si="30">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H20:H52" ca="1" si="30">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I20" s="34"/>
@@ -4753,26 +4850,26 @@
       <c r="CM20" s="34"/>
       <c r="CN20" s="34"/>
     </row>
-    <row r="21" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="81"/>
+    <row r="21" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A21" s="112"/>
       <c r="B21" s="36" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C21" s="37"/>
       <c r="D21" s="38">
         <v>0.33</v>
       </c>
-      <c r="E21" s="92">
+      <c r="E21" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F21" s="92">
+      <c r="F21" s="91">
         <f>E21+58</f>
         <v>46122</v>
       </c>
       <c r="G21" s="14"/>
       <c r="H21" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>59</v>
       </c>
       <c r="I21" s="39"/>
@@ -4860,18 +4957,18 @@
       <c r="CM21" s="39"/>
       <c r="CN21" s="39"/>
     </row>
-    <row r="22" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="81"/>
+    <row r="22" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A22" s="112"/>
       <c r="B22" s="36" t="s">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="C22" s="37"/>
       <c r="D22" s="38"/>
-      <c r="E22" s="92">
+      <c r="E22" s="91">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F22" s="92">
+      <c r="F22" s="91">
         <f>E22+58</f>
         <v>46122</v>
       </c>
@@ -4962,26 +5059,26 @@
       <c r="CM22" s="39"/>
       <c r="CN22" s="39"/>
     </row>
-    <row r="23" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="81"/>
+    <row r="23" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A23" s="112"/>
       <c r="B23" s="40" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="C23" s="41"/>
       <c r="D23" s="42">
         <v>0.33</v>
       </c>
-      <c r="E23" s="92">
+      <c r="E23" s="91">
         <f>F22+1</f>
         <v>46123</v>
       </c>
-      <c r="F23" s="93">
+      <c r="F23" s="92">
         <f>E23+7</f>
         <v>46130</v>
       </c>
       <c r="G23" s="14"/>
       <c r="H23" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I23" s="39"/>
@@ -5069,41 +5166,41 @@
       <c r="CM23" s="39"/>
       <c r="CN23" s="39"/>
     </row>
-    <row r="24" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="81"/>
+    <row r="24" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A24" s="112"/>
       <c r="B24" s="44" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46"/>
-      <c r="E24" s="94"/>
-      <c r="F24" s="95"/>
+      <c r="E24" s="93"/>
+      <c r="F24" s="94"/>
       <c r="G24" s="14"/>
       <c r="H24" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="81"/>
+    <row r="25" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A25" s="112"/>
       <c r="B25" s="47" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="49">
         <v>1</v>
       </c>
-      <c r="E25" s="96">
+      <c r="E25" s="95">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F25" s="96">
+      <c r="F25" s="95">
         <f>E25+20</f>
         <v>46084</v>
       </c>
       <c r="G25" s="14"/>
       <c r="H25" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>21</v>
       </c>
       <c r="I25" s="39"/>
@@ -5191,26 +5288,26 @@
       <c r="CM25" s="39"/>
       <c r="CN25" s="39"/>
     </row>
-    <row r="26" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A26" s="12"/>
       <c r="B26" s="47" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C26" s="48"/>
       <c r="D26" s="49">
         <v>0.8</v>
       </c>
-      <c r="E26" s="96">
+      <c r="E26" s="95">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F26" s="96">
+      <c r="F26" s="95">
         <f>E26+9</f>
         <v>46073</v>
       </c>
       <c r="G26" s="14"/>
       <c r="H26" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>10</v>
       </c>
       <c r="I26" s="39"/>
@@ -5298,25 +5395,25 @@
       <c r="CM26" s="39"/>
       <c r="CN26" s="39"/>
     </row>
-    <row r="27" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A27" s="12"/>
       <c r="B27" s="47" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C27" s="48"/>
       <c r="D27" s="49">
         <v>1</v>
       </c>
-      <c r="E27" s="96">
+      <c r="E27" s="95">
         <v>46083</v>
       </c>
-      <c r="F27" s="96">
+      <c r="F27" s="95">
         <f>E27+10</f>
         <v>46093</v>
       </c>
       <c r="G27" s="14"/>
       <c r="H27" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>11</v>
       </c>
       <c r="I27" s="39"/>
@@ -5404,26 +5501,26 @@
       <c r="CM27" s="39"/>
       <c r="CN27" s="39"/>
     </row>
-    <row r="28" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A28" s="12"/>
       <c r="B28" s="47" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C28" s="48"/>
       <c r="D28" s="49">
         <v>1</v>
       </c>
-      <c r="E28" s="96">
+      <c r="E28" s="95">
         <f>F27+1</f>
         <v>46094</v>
       </c>
-      <c r="F28" s="96">
+      <c r="F28" s="95">
         <f>E28+7</f>
         <v>46101</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I28" s="39"/>
@@ -5511,26 +5608,26 @@
       <c r="CM28" s="39"/>
       <c r="CN28" s="39"/>
     </row>
-    <row r="29" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A29" s="12"/>
       <c r="B29" s="47" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C29" s="48"/>
       <c r="D29" s="49">
         <v>1</v>
       </c>
-      <c r="E29" s="96">
+      <c r="E29" s="95">
         <f>E28</f>
         <v>46094</v>
       </c>
-      <c r="F29" s="96">
+      <c r="F29" s="95">
         <f>E29+7</f>
         <v>46101</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I29" s="39"/>
@@ -5618,20 +5715,20 @@
       <c r="CM29" s="39"/>
       <c r="CN29" s="39"/>
     </row>
-    <row r="30" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A30" s="12"/>
       <c r="B30" s="47" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="C30" s="48"/>
       <c r="D30" s="49">
         <v>1</v>
       </c>
-      <c r="E30" s="96">
+      <c r="E30" s="95">
         <f>F28+1</f>
         <v>46102</v>
       </c>
-      <c r="F30" s="96">
+      <c r="F30" s="95">
         <f>E30+7</f>
         <v>46109</v>
       </c>
@@ -5722,26 +5819,26 @@
       <c r="CM30" s="39"/>
       <c r="CN30" s="39"/>
     </row>
-    <row r="31" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A31" s="12"/>
       <c r="B31" s="47" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C31" s="48"/>
       <c r="D31" s="49">
         <v>1</v>
       </c>
-      <c r="E31" s="96">
+      <c r="E31" s="95">
         <f>F29+1</f>
         <v>46102</v>
       </c>
-      <c r="F31" s="96">
+      <c r="F31" s="95">
         <f>E31+7</f>
         <v>46109</v>
       </c>
       <c r="G31" s="14"/>
       <c r="H31" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I31" s="39"/>
@@ -5829,26 +5926,26 @@
       <c r="CM31" s="39"/>
       <c r="CN31" s="39"/>
     </row>
-    <row r="32" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A32" s="12"/>
       <c r="B32" s="47" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C32" s="48"/>
       <c r="D32" s="49">
         <v>0.15</v>
       </c>
-      <c r="E32" s="96">
+      <c r="E32" s="95">
         <f>F31+1</f>
         <v>46110</v>
       </c>
-      <c r="F32" s="96">
+      <c r="F32" s="95">
         <f>E32+3</f>
         <v>46113</v>
       </c>
       <c r="G32" s="14"/>
       <c r="H32" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>4</v>
       </c>
       <c r="I32" s="39"/>
@@ -5936,26 +6033,26 @@
       <c r="CM32" s="39"/>
       <c r="CN32" s="39"/>
     </row>
-    <row r="33" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A33" s="12"/>
       <c r="B33" s="47" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C33" s="48"/>
       <c r="D33" s="49">
         <v>0</v>
       </c>
-      <c r="E33" s="96">
+      <c r="E33" s="95">
         <f>F32+1</f>
         <v>46114</v>
       </c>
-      <c r="F33" s="96">
+      <c r="F33" s="95">
         <f>E33+8</f>
         <v>46122</v>
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>9</v>
       </c>
       <c r="I33" s="39"/>
@@ -6043,26 +6140,26 @@
       <c r="CM33" s="39"/>
       <c r="CN33" s="39"/>
     </row>
-    <row r="34" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A34" s="12"/>
       <c r="B34" s="47" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="C34" s="48"/>
       <c r="D34" s="49">
         <v>0</v>
       </c>
-      <c r="E34" s="96">
+      <c r="E34" s="95">
         <f>F32+1</f>
         <v>46114</v>
       </c>
-      <c r="F34" s="96">
+      <c r="F34" s="95">
         <f>E34+7</f>
         <v>46121</v>
       </c>
       <c r="G34" s="14"/>
       <c r="H34" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I34" s="39"/>
@@ -6150,26 +6247,26 @@
       <c r="CM34" s="39"/>
       <c r="CN34" s="39"/>
     </row>
-    <row r="35" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A35" s="12"/>
       <c r="B35" s="47" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="C35" s="48"/>
       <c r="D35" s="49">
         <v>0</v>
       </c>
-      <c r="E35" s="96">
+      <c r="E35" s="95">
         <f>F33+1</f>
         <v>46123</v>
       </c>
-      <c r="F35" s="96">
+      <c r="F35" s="95">
         <f>E35+7</f>
         <v>46130</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I35" s="39"/>
@@ -6257,18 +6354,18 @@
       <c r="CM35" s="39"/>
       <c r="CN35" s="39"/>
     </row>
-    <row r="36" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A36" s="12"/>
       <c r="B36" s="50" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="C36" s="51"/>
       <c r="D36" s="52"/>
-      <c r="E36" s="97"/>
-      <c r="F36" s="98"/>
+      <c r="E36" s="96"/>
+      <c r="F36" s="97"/>
       <c r="G36" s="14"/>
       <c r="H36" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I36" s="53"/>
@@ -6356,26 +6453,26 @@
       <c r="CM36" s="53"/>
       <c r="CN36" s="53"/>
     </row>
-    <row r="37" spans="1:92" s="35" customFormat="1" ht="68" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:92" s="35" customFormat="1" ht="68.099999999999994" customHeight="1" thickBot="1">
       <c r="A37" s="12"/>
-      <c r="B37" s="109" t="s">
-        <v>43</v>
+      <c r="B37" s="108" t="s">
+        <v>36</v>
       </c>
       <c r="C37" s="55"/>
       <c r="D37" s="56">
         <v>0.2</v>
       </c>
-      <c r="E37" s="99">
+      <c r="E37" s="98">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F37" s="99">
+      <c r="F37" s="98">
         <f>E37+14</f>
         <v>46078</v>
       </c>
       <c r="G37" s="14"/>
       <c r="H37" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>15</v>
       </c>
       <c r="I37" s="39"/>
@@ -6463,26 +6560,26 @@
       <c r="CM37" s="39"/>
       <c r="CN37" s="39"/>
     </row>
-    <row r="38" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A38" s="12"/>
       <c r="B38" s="54" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C38" s="55"/>
       <c r="D38" s="56">
         <v>0.2</v>
       </c>
-      <c r="E38" s="99">
+      <c r="E38" s="98">
         <f>F37+1</f>
         <v>46079</v>
       </c>
-      <c r="F38" s="99">
+      <c r="F38" s="98">
         <f>F35</f>
         <v>46130</v>
       </c>
       <c r="G38" s="14"/>
       <c r="H38" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>52</v>
       </c>
       <c r="I38" s="39"/>
@@ -6570,18 +6667,18 @@
       <c r="CM38" s="39"/>
       <c r="CN38" s="39"/>
     </row>
-    <row r="39" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A39" s="12"/>
       <c r="B39" s="50" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C39" s="51"/>
       <c r="D39" s="52"/>
-      <c r="E39" s="97"/>
-      <c r="F39" s="98"/>
+      <c r="E39" s="96"/>
+      <c r="F39" s="97"/>
       <c r="G39" s="14"/>
       <c r="H39" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I39" s="53"/>
@@ -6669,28 +6766,28 @@
       <c r="CM39" s="53"/>
       <c r="CN39" s="53"/>
     </row>
-    <row r="40" spans="1:92" s="35" customFormat="1" ht="43" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:92" s="35" customFormat="1" ht="42.95" thickBot="1">
       <c r="A40" s="12"/>
-      <c r="B40" s="109" t="s">
-        <v>45</v>
+      <c r="B40" s="108" t="s">
+        <v>39</v>
       </c>
       <c r="C40" s="55"/>
       <c r="D40" s="56">
         <v>0.9</v>
       </c>
-      <c r="E40" s="99">
+      <c r="E40" s="98">
         <f>Project_Start</f>
         <v>46064</v>
       </c>
-      <c r="F40" s="99">
+      <c r="F40" s="98">
         <f>E40+21</f>
         <v>46085</v>
       </c>
-      <c r="G40" s="111" t="s">
-        <v>64</v>
+      <c r="G40" s="110" t="s">
+        <v>40</v>
       </c>
       <c r="H40" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>22</v>
       </c>
       <c r="I40" s="39"/>
@@ -6778,26 +6875,26 @@
       <c r="CM40" s="39"/>
       <c r="CN40" s="39"/>
     </row>
-    <row r="41" spans="1:92" s="35" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:92" s="35" customFormat="1" ht="24" customHeight="1" thickBot="1">
       <c r="A41" s="12"/>
-      <c r="B41" s="109" t="s">
-        <v>55</v>
+      <c r="B41" s="108" t="s">
+        <v>41</v>
       </c>
       <c r="C41" s="55"/>
       <c r="D41" s="56">
         <v>0.3</v>
       </c>
-      <c r="E41" s="99">
+      <c r="E41" s="98">
         <f>F40</f>
         <v>46085</v>
       </c>
-      <c r="F41" s="99">
+      <c r="F41" s="98">
         <f>F35</f>
         <v>46130</v>
       </c>
       <c r="G41" s="14"/>
       <c r="H41" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>46</v>
       </c>
       <c r="I41" s="39"/>
@@ -6885,20 +6982,20 @@
       <c r="CM41" s="39"/>
       <c r="CN41" s="39"/>
     </row>
-    <row r="42" spans="1:92" s="35" customFormat="1" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:92" s="35" customFormat="1" ht="35.1" customHeight="1" thickBot="1">
       <c r="A42" s="12"/>
       <c r="B42" s="54" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="C42" s="55"/>
       <c r="D42" s="56">
         <v>1</v>
       </c>
-      <c r="E42" s="99">
+      <c r="E42" s="98">
         <f>F40</f>
         <v>46085</v>
       </c>
-      <c r="F42" s="99">
+      <c r="F42" s="98">
         <f>F35</f>
         <v>46130</v>
       </c>
@@ -6989,20 +7086,20 @@
       <c r="CM42" s="39"/>
       <c r="CN42" s="39"/>
     </row>
-    <row r="43" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A43" s="12"/>
       <c r="B43" s="54" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C43" s="55"/>
       <c r="D43" s="56">
         <v>0</v>
       </c>
-      <c r="E43" s="99"/>
-      <c r="F43" s="99"/>
+      <c r="E43" s="98"/>
+      <c r="F43" s="98"/>
       <c r="G43" s="14"/>
       <c r="H43" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I43" s="39"/>
@@ -7090,18 +7187,18 @@
       <c r="CM43" s="39"/>
       <c r="CN43" s="39"/>
     </row>
-    <row r="44" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A44" s="12"/>
       <c r="B44" s="57" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C44" s="58"/>
       <c r="D44" s="59"/>
-      <c r="E44" s="100"/>
-      <c r="F44" s="101"/>
+      <c r="E44" s="99"/>
+      <c r="F44" s="100"/>
       <c r="G44" s="14"/>
       <c r="H44" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I44" s="60"/>
@@ -7189,26 +7286,26 @@
       <c r="CM44" s="60"/>
       <c r="CN44" s="60"/>
     </row>
-    <row r="45" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A45" s="12"/>
       <c r="B45" s="61" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C45" s="62"/>
       <c r="D45" s="63">
         <v>1</v>
       </c>
-      <c r="E45" s="102">
+      <c r="E45" s="101">
         <f>E37</f>
         <v>46064</v>
       </c>
-      <c r="F45" s="102">
+      <c r="F45" s="101">
         <f>E49-3</f>
         <v>46157</v>
       </c>
       <c r="G45" s="14"/>
       <c r="H45" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>94</v>
       </c>
       <c r="I45" s="39"/>
@@ -7296,25 +7393,25 @@
       <c r="CM45" s="39"/>
       <c r="CN45" s="39"/>
     </row>
-    <row r="46" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A46" s="12"/>
       <c r="B46" s="61" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C46" s="62"/>
       <c r="D46" s="63">
         <v>0.9</v>
       </c>
-      <c r="E46" s="102">
+      <c r="E46" s="101">
         <v>46146</v>
       </c>
-      <c r="F46" s="102">
+      <c r="F46" s="101">
         <f>E46+7</f>
         <v>46153</v>
       </c>
       <c r="G46" s="14"/>
       <c r="H46" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I46" s="39"/>
@@ -7402,7 +7499,7 @@
       <c r="CM46" s="39"/>
       <c r="CN46" s="39"/>
     </row>
-    <row r="47" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A47" s="12"/>
       <c r="B47" s="61" t="s">
         <v>47</v>
@@ -7411,16 +7508,16 @@
       <c r="D47" s="63">
         <v>0</v>
       </c>
-      <c r="E47" s="102">
+      <c r="E47" s="101">
         <v>46146</v>
       </c>
-      <c r="F47" s="102">
+      <c r="F47" s="101">
         <f>E47+7</f>
         <v>46153</v>
       </c>
       <c r="G47" s="14"/>
       <c r="H47" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I47" s="39"/>
@@ -7508,7 +7605,7 @@
       <c r="CM47" s="39"/>
       <c r="CN47" s="39"/>
     </row>
-    <row r="48" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A48" s="12"/>
       <c r="B48" s="61" t="s">
         <v>48</v>
@@ -7517,17 +7614,17 @@
       <c r="D48" s="63">
         <v>0</v>
       </c>
-      <c r="E48" s="102">
+      <c r="E48" s="101">
         <f>F47</f>
         <v>46153</v>
       </c>
-      <c r="F48" s="102">
+      <c r="F48" s="101">
         <f>E48+7</f>
         <v>46160</v>
       </c>
       <c r="G48" s="14"/>
       <c r="H48" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I48" s="39"/>
@@ -7615,7 +7712,7 @@
       <c r="CM48" s="39"/>
       <c r="CN48" s="39"/>
     </row>
-    <row r="49" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A49" s="12"/>
       <c r="B49" s="61" t="s">
         <v>49</v>
@@ -7624,17 +7721,17 @@
       <c r="D49" s="63">
         <v>0</v>
       </c>
-      <c r="E49" s="102">
+      <c r="E49" s="101">
         <f>F48</f>
         <v>46160</v>
       </c>
-      <c r="F49" s="102">
+      <c r="F49" s="101">
         <f>E49+7</f>
         <v>46167</v>
       </c>
       <c r="G49" s="14"/>
       <c r="H49" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>8</v>
       </c>
       <c r="I49" s="39"/>
@@ -7722,7 +7819,7 @@
       <c r="CM49" s="39"/>
       <c r="CN49" s="39"/>
     </row>
-    <row r="50" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A50" s="12"/>
       <c r="B50" s="61" t="s">
         <v>50</v>
@@ -7731,17 +7828,17 @@
       <c r="D50" s="63">
         <v>0</v>
       </c>
-      <c r="E50" s="102">
+      <c r="E50" s="101">
         <f>F49</f>
         <v>46167</v>
       </c>
-      <c r="F50" s="102">
+      <c r="F50" s="101">
         <f>E50+14</f>
         <v>46181</v>
       </c>
       <c r="G50" s="14"/>
       <c r="H50" s="4">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v>15</v>
       </c>
       <c r="I50" s="39"/>
@@ -7829,18 +7926,18 @@
       <c r="CM50" s="39"/>
       <c r="CN50" s="39"/>
     </row>
-    <row r="51" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A51" s="12"/>
       <c r="B51" s="64" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C51" s="65"/>
       <c r="D51" s="66"/>
-      <c r="E51" s="103"/>
-      <c r="F51" s="103"/>
+      <c r="E51" s="102"/>
+      <c r="F51" s="102"/>
       <c r="G51" s="14"/>
       <c r="H51" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I51" s="34"/>
@@ -7928,18 +8025,18 @@
       <c r="CM51" s="34"/>
       <c r="CN51" s="34"/>
     </row>
-    <row r="52" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="81"/>
+    <row r="52" spans="1:92" s="35" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A52" s="112"/>
       <c r="B52" s="67" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C52" s="68"/>
       <c r="D52" s="69"/>
-      <c r="E52" s="104"/>
-      <c r="F52" s="105"/>
+      <c r="E52" s="103"/>
+      <c r="F52" s="104"/>
       <c r="G52" s="14"/>
       <c r="H52" s="5" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ca="1" si="30"/>
         <v/>
       </c>
       <c r="I52" s="70"/>
@@ -8027,24 +8124,18 @@
       <c r="CM52" s="70"/>
       <c r="CN52" s="70"/>
     </row>
-    <row r="53" spans="1:92" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:92" ht="30" customHeight="1">
       <c r="G53" s="2"/>
     </row>
-    <row r="54" spans="1:92" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:92" ht="30" customHeight="1">
       <c r="C54" s="13"/>
-      <c r="F54" s="108"/>
+      <c r="F54" s="107"/>
     </row>
-    <row r="55" spans="1:92" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:92" ht="30" customHeight="1">
       <c r="C55" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="CH4:CN4"/>
     <mergeCell ref="Q2:Z2"/>
     <mergeCell ref="Q1:Z1"/>
@@ -8061,6 +8152,12 @@
     <mergeCell ref="BM4:BS4"/>
     <mergeCell ref="BT4:BZ4"/>
     <mergeCell ref="CA4:CG4"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D52">
     <cfRule type="dataBar" priority="102">
@@ -8372,110 +8469,110 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.95"/>
   <cols>
     <col min="1" max="1" width="87" style="6" customWidth="1"/>
     <col min="2" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="2" spans="1:2" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:2" ht="46.5" customHeight="1"/>
+    <row r="2" spans="1:2" s="8" customFormat="1" ht="15.95">
       <c r="A2" s="74" t="s">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="B2" s="7"/>
     </row>
-    <row r="3" spans="1:2" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:2" s="10" customFormat="1" ht="27" customHeight="1">
       <c r="A3" s="75"/>
       <c r="B3" s="11"/>
     </row>
-    <row r="4" spans="1:2" s="9" customFormat="1" ht="31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" s="9" customFormat="1" ht="30.95">
       <c r="A4" s="76" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="74.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:2" ht="74.25" customHeight="1">
       <c r="A5" s="77" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:2" ht="26.25" customHeight="1">
       <c r="A6" s="76" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="6" customFormat="1" ht="205.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:2" s="6" customFormat="1" ht="205.35" customHeight="1">
       <c r="A7" s="78" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="9" customFormat="1" ht="31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" s="9" customFormat="1" ht="30.95">
       <c r="A8" s="76" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="60" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:2" ht="60">
       <c r="A9" s="77" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="6" customFormat="1" ht="28.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:2" s="6" customFormat="1" ht="28.35" customHeight="1">
       <c r="A10" s="79" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="9" customFormat="1" ht="31" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" s="9" customFormat="1" ht="30.95">
       <c r="A11" s="76" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:2" ht="30">
       <c r="A12" s="77" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="6" customFormat="1" ht="28.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:2" s="6" customFormat="1" ht="28.35" customHeight="1">
       <c r="A13" s="79" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="9" customFormat="1" ht="31" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" s="9" customFormat="1" ht="30.95">
       <c r="A14" s="76" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:2" ht="75" customHeight="1">
       <c r="A15" s="77" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:2" ht="75">
       <c r="A16" s="77" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:1">
       <c r="A17" s="80"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:1">
       <c r="A18" s="80"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:1">
       <c r="A19" s="80"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:1">
       <c r="A20" s="80"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:1">
       <c r="A21" s="80"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:1">
       <c r="A22" s="80"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:1">
       <c r="A23" s="80"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:1">
       <c r="A24" s="80"/>
     </row>
   </sheetData>
@@ -8491,6 +8588,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -8802,74 +8928,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2348D59-3426-404A-A0C5-6456F6613EDB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2348D59-3426-404A-A0C5-6456F6613EDB}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>